<commit_message>
Organized result data and sign agreement
Created a result struct for saving different heats and temperatures. Changed the ecuations to follow sign agreements.
</commit_message>
<xml_diff>
--- a/teidecode_v1/Thermal_Data.xlsx
+++ b/teidecode_v1/Thermal_Data.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduardo Navarro\Desktop\Cosas\Teidesat\Nueva carpeta\TeideThermal\teidecode_v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF56F914-63FC-4545-8856-CE21525E64FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9328060-3922-4B4F-9519-0E5D671A65AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2531,10 +2531,6 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="17" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -2612,6 +2608,10 @@
     <xf numFmtId="0" fontId="1" fillId="21" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10003,10 +10003,10 @@
         <v>149</v>
       </c>
       <c r="G2" s="32"/>
-      <c r="H2" s="118" t="s">
+      <c r="H2" s="147" t="s">
         <v>150</v>
       </c>
-      <c r="I2" s="119"/>
+      <c r="I2" s="148"/>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="33" t="s">
@@ -11021,24 +11021,24 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:6" ht="45">
-      <c r="B2" s="146" t="s">
+      <c r="B2" s="144" t="s">
         <v>266</v>
       </c>
-      <c r="C2" s="147" t="s">
+      <c r="C2" s="145" t="s">
         <v>267</v>
       </c>
-      <c r="D2" s="147" t="s">
+      <c r="D2" s="145" t="s">
         <v>265</v>
       </c>
-      <c r="E2" s="147" t="s">
+      <c r="E2" s="145" t="s">
         <v>264</v>
       </c>
-      <c r="F2" s="148" t="s">
+      <c r="F2" s="146" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1">
-      <c r="B3" s="136">
+      <c r="B3" s="134">
         <v>1</v>
       </c>
       <c r="C3" s="85">
@@ -11048,9 +11048,9 @@
         <v>0</v>
       </c>
       <c r="E3" s="85">
-        <v>0</v>
-      </c>
-      <c r="F3" s="137">
+        <v>300</v>
+      </c>
+      <c r="F3" s="135">
         <v>1</v>
       </c>
     </row>
@@ -11069,7 +11069,7 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1"/>
     <row r="2" spans="1:14" ht="15.75" thickBot="1">
-      <c r="B2" s="141" t="s">
+      <c r="B2" s="139" t="s">
         <v>257</v>
       </c>
       <c r="C2" s="87" t="s">
@@ -11078,13 +11078,13 @@
       <c r="D2" s="86" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="125" t="s">
+      <c r="E2" s="123" t="s">
         <v>260</v>
       </c>
       <c r="F2" s="93" t="s">
         <v>259</v>
       </c>
-      <c r="G2" s="126"/>
+      <c r="G2" s="124"/>
     </row>
     <row r="3" spans="1:14">
       <c r="B3" s="89" t="s">
@@ -11156,13 +11156,13 @@
       <c r="G6" s="96"/>
     </row>
     <row r="7" spans="1:14">
-      <c r="B7" s="120" t="s">
+      <c r="B7" s="118" t="s">
         <v>261</v>
       </c>
-      <c r="C7" s="121"/>
-      <c r="D7" s="122"/>
-      <c r="E7" s="123"/>
-      <c r="F7" s="124"/>
+      <c r="C7" s="119"/>
+      <c r="D7" s="120"/>
+      <c r="E7" s="121"/>
+      <c r="F7" s="122"/>
       <c r="G7" s="96"/>
     </row>
     <row r="8" spans="1:14">
@@ -12053,58 +12053,58 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:15" ht="15.75" thickBot="1">
-      <c r="B2" s="142" t="s">
+      <c r="B2" s="140" t="s">
         <v>257</v>
       </c>
-      <c r="C2" s="127" t="s">
+      <c r="C2" s="125" t="s">
         <v>260</v>
       </c>
-      <c r="D2" s="128" t="s">
+      <c r="D2" s="126" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="128" t="s">
+      <c r="E2" s="126" t="s">
         <v>259</v>
       </c>
-      <c r="F2" s="129"/>
-      <c r="G2" s="129"/>
-      <c r="H2" s="129"/>
-      <c r="I2" s="129"/>
-      <c r="J2" s="129"/>
-      <c r="K2" s="129"/>
-      <c r="L2" s="129"/>
-      <c r="M2" s="129"/>
-      <c r="N2" s="129"/>
-      <c r="O2" s="130"/>
+      <c r="F2" s="127"/>
+      <c r="G2" s="127"/>
+      <c r="H2" s="127"/>
+      <c r="I2" s="127"/>
+      <c r="J2" s="127"/>
+      <c r="K2" s="127"/>
+      <c r="L2" s="127"/>
+      <c r="M2" s="127"/>
+      <c r="N2" s="127"/>
+      <c r="O2" s="128"/>
     </row>
     <row r="3" spans="2:15">
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="141" t="s">
         <v>214</v>
       </c>
-      <c r="C3" s="131">
-        <v>0</v>
-      </c>
-      <c r="D3" s="132">
-        <v>0</v>
-      </c>
-      <c r="E3" s="132">
-        <v>0</v>
-      </c>
-      <c r="F3" s="132"/>
-      <c r="G3" s="132"/>
-      <c r="H3" s="132"/>
-      <c r="I3" s="132"/>
-      <c r="J3" s="132"/>
-      <c r="K3" s="132"/>
-      <c r="L3" s="132"/>
-      <c r="M3" s="132"/>
-      <c r="N3" s="132"/>
-      <c r="O3" s="133"/>
+      <c r="C3" s="129">
+        <v>0</v>
+      </c>
+      <c r="D3" s="130">
+        <v>0</v>
+      </c>
+      <c r="E3" s="130">
+        <v>0</v>
+      </c>
+      <c r="F3" s="130"/>
+      <c r="G3" s="130"/>
+      <c r="H3" s="130"/>
+      <c r="I3" s="130"/>
+      <c r="J3" s="130"/>
+      <c r="K3" s="130"/>
+      <c r="L3" s="130"/>
+      <c r="M3" s="130"/>
+      <c r="N3" s="130"/>
+      <c r="O3" s="131"/>
     </row>
     <row r="4" spans="2:15">
-      <c r="B4" s="144" t="s">
+      <c r="B4" s="142" t="s">
         <v>215</v>
       </c>
-      <c r="C4" s="134">
+      <c r="C4" s="132">
         <v>0</v>
       </c>
       <c r="D4" s="84">
@@ -12122,13 +12122,13 @@
       <c r="L4" s="84"/>
       <c r="M4" s="84"/>
       <c r="N4" s="84"/>
-      <c r="O4" s="135"/>
+      <c r="O4" s="133"/>
     </row>
     <row r="5" spans="2:15">
-      <c r="B5" s="144" t="s">
+      <c r="B5" s="142" t="s">
         <v>216</v>
       </c>
-      <c r="C5" s="134">
+      <c r="C5" s="132">
         <v>0</v>
       </c>
       <c r="D5" s="84">
@@ -12146,13 +12146,13 @@
       <c r="L5" s="84"/>
       <c r="M5" s="84"/>
       <c r="N5" s="84"/>
-      <c r="O5" s="135"/>
+      <c r="O5" s="133"/>
     </row>
     <row r="6" spans="2:15">
-      <c r="B6" s="144" t="s">
+      <c r="B6" s="142" t="s">
         <v>217</v>
       </c>
-      <c r="C6" s="134">
+      <c r="C6" s="132">
         <v>0</v>
       </c>
       <c r="D6" s="84">
@@ -12170,13 +12170,13 @@
       <c r="L6" s="84"/>
       <c r="M6" s="84"/>
       <c r="N6" s="84"/>
-      <c r="O6" s="135"/>
+      <c r="O6" s="133"/>
     </row>
     <row r="7" spans="2:15">
-      <c r="B7" s="144" t="s">
+      <c r="B7" s="142" t="s">
         <v>218</v>
       </c>
-      <c r="C7" s="134">
+      <c r="C7" s="132">
         <v>0</v>
       </c>
       <c r="D7" s="84">
@@ -12194,13 +12194,13 @@
       <c r="L7" s="84"/>
       <c r="M7" s="84"/>
       <c r="N7" s="84"/>
-      <c r="O7" s="135"/>
+      <c r="O7" s="133"/>
     </row>
     <row r="8" spans="2:15">
-      <c r="B8" s="144" t="s">
+      <c r="B8" s="142" t="s">
         <v>219</v>
       </c>
-      <c r="C8" s="134">
+      <c r="C8" s="132">
         <v>0</v>
       </c>
       <c r="D8" s="84">
@@ -12218,13 +12218,13 @@
       <c r="L8" s="84"/>
       <c r="M8" s="84"/>
       <c r="N8" s="84"/>
-      <c r="O8" s="135"/>
+      <c r="O8" s="133"/>
     </row>
     <row r="9" spans="2:15">
-      <c r="B9" s="144" t="s">
+      <c r="B9" s="142" t="s">
         <v>220</v>
       </c>
-      <c r="C9" s="134">
+      <c r="C9" s="132">
         <v>0</v>
       </c>
       <c r="D9" s="84">
@@ -12242,13 +12242,13 @@
       <c r="L9" s="84"/>
       <c r="M9" s="84"/>
       <c r="N9" s="84"/>
-      <c r="O9" s="135"/>
+      <c r="O9" s="133"/>
     </row>
     <row r="10" spans="2:15">
-      <c r="B10" s="144" t="s">
+      <c r="B10" s="142" t="s">
         <v>221</v>
       </c>
-      <c r="C10" s="134">
+      <c r="C10" s="132">
         <v>0</v>
       </c>
       <c r="D10" s="84">
@@ -12266,13 +12266,13 @@
       <c r="L10" s="84"/>
       <c r="M10" s="84"/>
       <c r="N10" s="84"/>
-      <c r="O10" s="135"/>
+      <c r="O10" s="133"/>
     </row>
     <row r="11" spans="2:15">
-      <c r="B11" s="144" t="s">
+      <c r="B11" s="142" t="s">
         <v>222</v>
       </c>
-      <c r="C11" s="134">
+      <c r="C11" s="132">
         <v>0</v>
       </c>
       <c r="D11" s="84">
@@ -12290,13 +12290,13 @@
       <c r="L11" s="84"/>
       <c r="M11" s="84"/>
       <c r="N11" s="84"/>
-      <c r="O11" s="135"/>
+      <c r="O11" s="133"/>
     </row>
     <row r="12" spans="2:15">
-      <c r="B12" s="144" t="s">
+      <c r="B12" s="142" t="s">
         <v>223</v>
       </c>
-      <c r="C12" s="134">
+      <c r="C12" s="132">
         <v>0</v>
       </c>
       <c r="D12" s="84">
@@ -12314,13 +12314,13 @@
       <c r="L12" s="84"/>
       <c r="M12" s="84"/>
       <c r="N12" s="84"/>
-      <c r="O12" s="135"/>
+      <c r="O12" s="133"/>
     </row>
     <row r="13" spans="2:15">
-      <c r="B13" s="144" t="s">
+      <c r="B13" s="142" t="s">
         <v>224</v>
       </c>
-      <c r="C13" s="134">
+      <c r="C13" s="132">
         <v>0</v>
       </c>
       <c r="D13" s="84">
@@ -12338,13 +12338,13 @@
       <c r="L13" s="84"/>
       <c r="M13" s="84"/>
       <c r="N13" s="84"/>
-      <c r="O13" s="135"/>
+      <c r="O13" s="133"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="144" t="s">
+      <c r="B14" s="142" t="s">
         <v>225</v>
       </c>
-      <c r="C14" s="134">
+      <c r="C14" s="132">
         <v>0</v>
       </c>
       <c r="D14" s="84">
@@ -12362,13 +12362,13 @@
       <c r="L14" s="84"/>
       <c r="M14" s="84"/>
       <c r="N14" s="84"/>
-      <c r="O14" s="135"/>
+      <c r="O14" s="133"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="144" t="s">
+      <c r="B15" s="142" t="s">
         <v>226</v>
       </c>
-      <c r="C15" s="134">
+      <c r="C15" s="132">
         <v>0</v>
       </c>
       <c r="D15" s="84">
@@ -12386,13 +12386,13 @@
       <c r="L15" s="84"/>
       <c r="M15" s="84"/>
       <c r="N15" s="84"/>
-      <c r="O15" s="135"/>
+      <c r="O15" s="133"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="144" t="s">
+      <c r="B16" s="142" t="s">
         <v>227</v>
       </c>
-      <c r="C16" s="134">
+      <c r="C16" s="132">
         <v>0</v>
       </c>
       <c r="D16" s="84">
@@ -12410,13 +12410,13 @@
       <c r="L16" s="84"/>
       <c r="M16" s="84"/>
       <c r="N16" s="84"/>
-      <c r="O16" s="135"/>
+      <c r="O16" s="133"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="144" t="s">
+      <c r="B17" s="142" t="s">
         <v>228</v>
       </c>
-      <c r="C17" s="134">
+      <c r="C17" s="132">
         <v>0</v>
       </c>
       <c r="D17" s="84">
@@ -12434,13 +12434,13 @@
       <c r="L17" s="84"/>
       <c r="M17" s="84"/>
       <c r="N17" s="84"/>
-      <c r="O17" s="135"/>
+      <c r="O17" s="133"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="144" t="s">
+      <c r="B18" s="142" t="s">
         <v>229</v>
       </c>
-      <c r="C18" s="134">
+      <c r="C18" s="132">
         <v>0</v>
       </c>
       <c r="D18" s="84">
@@ -12458,13 +12458,13 @@
       <c r="L18" s="84"/>
       <c r="M18" s="84"/>
       <c r="N18" s="84"/>
-      <c r="O18" s="135"/>
+      <c r="O18" s="133"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="144" t="s">
+      <c r="B19" s="142" t="s">
         <v>230</v>
       </c>
-      <c r="C19" s="134">
+      <c r="C19" s="132">
         <v>0</v>
       </c>
       <c r="D19" s="84">
@@ -12482,13 +12482,13 @@
       <c r="L19" s="84"/>
       <c r="M19" s="84"/>
       <c r="N19" s="84"/>
-      <c r="O19" s="135"/>
+      <c r="O19" s="133"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="144" t="s">
+      <c r="B20" s="142" t="s">
         <v>231</v>
       </c>
-      <c r="C20" s="134">
+      <c r="C20" s="132">
         <v>0</v>
       </c>
       <c r="D20" s="84">
@@ -12506,13 +12506,13 @@
       <c r="L20" s="84"/>
       <c r="M20" s="84"/>
       <c r="N20" s="84"/>
-      <c r="O20" s="135"/>
+      <c r="O20" s="133"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="144" t="s">
+      <c r="B21" s="142" t="s">
         <v>232</v>
       </c>
-      <c r="C21" s="134">
+      <c r="C21" s="132">
         <v>0</v>
       </c>
       <c r="D21" s="84">
@@ -12530,13 +12530,13 @@
       <c r="L21" s="84"/>
       <c r="M21" s="84"/>
       <c r="N21" s="84"/>
-      <c r="O21" s="135"/>
+      <c r="O21" s="133"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="144" t="s">
+      <c r="B22" s="142" t="s">
         <v>233</v>
       </c>
-      <c r="C22" s="134">
+      <c r="C22" s="132">
         <v>0</v>
       </c>
       <c r="D22" s="84">
@@ -12554,13 +12554,13 @@
       <c r="L22" s="84"/>
       <c r="M22" s="84"/>
       <c r="N22" s="84"/>
-      <c r="O22" s="135"/>
+      <c r="O22" s="133"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="144" t="s">
+      <c r="B23" s="142" t="s">
         <v>234</v>
       </c>
-      <c r="C23" s="134">
+      <c r="C23" s="132">
         <v>0</v>
       </c>
       <c r="D23" s="84">
@@ -12578,13 +12578,13 @@
       <c r="L23" s="84"/>
       <c r="M23" s="84"/>
       <c r="N23" s="84"/>
-      <c r="O23" s="135"/>
+      <c r="O23" s="133"/>
     </row>
     <row r="24" spans="2:15">
-      <c r="B24" s="144" t="s">
+      <c r="B24" s="142" t="s">
         <v>235</v>
       </c>
-      <c r="C24" s="134">
+      <c r="C24" s="132">
         <v>0</v>
       </c>
       <c r="D24" s="84">
@@ -12602,13 +12602,13 @@
       <c r="L24" s="84"/>
       <c r="M24" s="84"/>
       <c r="N24" s="84"/>
-      <c r="O24" s="135"/>
+      <c r="O24" s="133"/>
     </row>
     <row r="25" spans="2:15">
-      <c r="B25" s="144" t="s">
+      <c r="B25" s="142" t="s">
         <v>236</v>
       </c>
-      <c r="C25" s="134">
+      <c r="C25" s="132">
         <v>0</v>
       </c>
       <c r="D25" s="84">
@@ -12626,13 +12626,13 @@
       <c r="L25" s="84"/>
       <c r="M25" s="84"/>
       <c r="N25" s="84"/>
-      <c r="O25" s="135"/>
+      <c r="O25" s="133"/>
     </row>
     <row r="26" spans="2:15">
-      <c r="B26" s="144" t="s">
+      <c r="B26" s="142" t="s">
         <v>237</v>
       </c>
-      <c r="C26" s="134">
+      <c r="C26" s="132">
         <v>0</v>
       </c>
       <c r="D26" s="84">
@@ -12650,13 +12650,13 @@
       <c r="L26" s="84"/>
       <c r="M26" s="84"/>
       <c r="N26" s="84"/>
-      <c r="O26" s="135"/>
+      <c r="O26" s="133"/>
     </row>
     <row r="27" spans="2:15">
-      <c r="B27" s="144" t="s">
+      <c r="B27" s="142" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="134">
+      <c r="C27" s="132">
         <v>0</v>
       </c>
       <c r="D27" s="84">
@@ -12674,13 +12674,13 @@
       <c r="L27" s="84"/>
       <c r="M27" s="84"/>
       <c r="N27" s="84"/>
-      <c r="O27" s="135"/>
+      <c r="O27" s="133"/>
     </row>
     <row r="28" spans="2:15">
-      <c r="B28" s="144" t="s">
+      <c r="B28" s="142" t="s">
         <v>239</v>
       </c>
-      <c r="C28" s="134">
+      <c r="C28" s="132">
         <v>0</v>
       </c>
       <c r="D28" s="84">
@@ -12698,13 +12698,13 @@
       <c r="L28" s="84"/>
       <c r="M28" s="84"/>
       <c r="N28" s="84"/>
-      <c r="O28" s="135"/>
+      <c r="O28" s="133"/>
     </row>
     <row r="29" spans="2:15">
-      <c r="B29" s="144" t="s">
+      <c r="B29" s="142" t="s">
         <v>240</v>
       </c>
-      <c r="C29" s="134">
+      <c r="C29" s="132">
         <v>0</v>
       </c>
       <c r="D29" s="84">
@@ -12722,13 +12722,13 @@
       <c r="L29" s="84"/>
       <c r="M29" s="84"/>
       <c r="N29" s="84"/>
-      <c r="O29" s="135"/>
+      <c r="O29" s="133"/>
     </row>
     <row r="30" spans="2:15">
-      <c r="B30" s="144" t="s">
+      <c r="B30" s="142" t="s">
         <v>241</v>
       </c>
-      <c r="C30" s="134">
+      <c r="C30" s="132">
         <v>0</v>
       </c>
       <c r="D30" s="84">
@@ -12746,31 +12746,31 @@
       <c r="L30" s="84"/>
       <c r="M30" s="84"/>
       <c r="N30" s="84"/>
-      <c r="O30" s="135"/>
+      <c r="O30" s="133"/>
     </row>
     <row r="31" spans="2:15">
-      <c r="B31" s="145" t="s">
+      <c r="B31" s="143" t="s">
         <v>242</v>
       </c>
-      <c r="C31" s="138">
-        <v>0</v>
-      </c>
-      <c r="D31" s="122">
-        <v>0</v>
-      </c>
-      <c r="E31" s="122">
-        <v>0</v>
-      </c>
-      <c r="F31" s="122"/>
-      <c r="G31" s="122"/>
-      <c r="H31" s="122"/>
-      <c r="I31" s="122"/>
-      <c r="J31" s="122"/>
-      <c r="K31" s="122"/>
-      <c r="L31" s="122"/>
-      <c r="M31" s="122"/>
-      <c r="N31" s="122"/>
-      <c r="O31" s="139"/>
+      <c r="C31" s="136">
+        <v>0</v>
+      </c>
+      <c r="D31" s="120">
+        <v>0</v>
+      </c>
+      <c r="E31" s="120">
+        <v>0</v>
+      </c>
+      <c r="F31" s="120"/>
+      <c r="G31" s="120"/>
+      <c r="H31" s="120"/>
+      <c r="I31" s="120"/>
+      <c r="J31" s="120"/>
+      <c r="K31" s="120"/>
+      <c r="L31" s="120"/>
+      <c r="M31" s="120"/>
+      <c r="N31" s="120"/>
+      <c r="O31" s="137"/>
     </row>
     <row r="32" spans="2:15">
       <c r="B32" s="96"/>
@@ -12811,7 +12811,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:13" ht="15.75" thickBot="1"/>
-    <row r="2" spans="2:13" ht="30" customHeight="1" thickBot="1">
+    <row r="2" spans="2:13" ht="46.5" customHeight="1" thickBot="1">
       <c r="B2" s="111" t="s">
         <v>252</v>
       </c>
@@ -12842,7 +12842,7 @@
       <c r="K2" s="113" t="s">
         <v>251</v>
       </c>
-      <c r="L2" s="140" t="s">
+      <c r="L2" s="138" t="s">
         <v>262</v>
       </c>
       <c r="M2" s="114" t="s">

</xml_diff>

<commit_message>
Added possibility to save data on excel
The data can be exported on excel now. Main restructured for most logical use.
</commit_message>
<xml_diff>
--- a/teidecode_v1/Thermal_Data.xlsx
+++ b/teidecode_v1/Thermal_Data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduardo Navarro\Desktop\Cosas\Teidesat\Nueva carpeta\TeideThermal\teidecode_v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9328060-3922-4B4F-9519-0E5D671A65AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB26D28-3013-4CD9-BC48-2EE9A94F7B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes properties" sheetId="1" r:id="rId1"/>
@@ -1274,11 +1274,18 @@
     <numFmt numFmtId="166" formatCode="#,##0.000000"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="11">
+  <fonts count="12">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1474,7 +1481,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="61">
+  <borders count="60">
     <border>
       <left/>
       <right/>
@@ -2015,19 +2022,6 @@
         <color indexed="64"/>
       </left>
       <right/>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
-      <right/>
       <top style="thin">
         <color indexed="64"/>
       </top>
@@ -2296,163 +2290,163 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="149">
+  <cellXfs count="146">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="6" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="8" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="3" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="4" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="4" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="5" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="4" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="4" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="5" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="4" fillId="14" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="5" fillId="14" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="10" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="13" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="13" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="3" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="3" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2461,34 +2455,19 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="40" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -2498,10 +2477,7 @@
     <xf numFmtId="0" fontId="0" fillId="18" borderId="33" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="23" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="40" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="39" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="37" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2509,57 +2485,54 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="47" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="48" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="50" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="49" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="19" borderId="51" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="17" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="17" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="54" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="43" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="42" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="57" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2568,50 +2541,62 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="56" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="55" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="27" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="44" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="46" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="45" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="58" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="60" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="40" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="18" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="21" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="44" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="41" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="18" borderId="58" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="21" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -10003,10 +9988,10 @@
         <v>149</v>
       </c>
       <c r="G2" s="32"/>
-      <c r="H2" s="147" t="s">
+      <c r="H2" s="140" t="s">
         <v>150</v>
       </c>
-      <c r="I2" s="148"/>
+      <c r="I2" s="141"/>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="33" t="s">
@@ -11021,24 +11006,24 @@
   <sheetData>
     <row r="1" spans="2:6" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:6" ht="45">
-      <c r="B2" s="144" t="s">
+      <c r="B2" s="137" t="s">
         <v>266</v>
       </c>
-      <c r="C2" s="145" t="s">
+      <c r="C2" s="138" t="s">
         <v>267</v>
       </c>
-      <c r="D2" s="145" t="s">
+      <c r="D2" s="138" t="s">
         <v>265</v>
       </c>
-      <c r="E2" s="145" t="s">
+      <c r="E2" s="138" t="s">
         <v>264</v>
       </c>
-      <c r="F2" s="146" t="s">
+      <c r="F2" s="139" t="s">
         <v>263</v>
       </c>
     </row>
     <row r="3" spans="2:6" ht="15.75" thickBot="1">
-      <c r="B3" s="134">
+      <c r="B3" s="127">
         <v>1</v>
       </c>
       <c r="C3" s="85">
@@ -11050,7 +11035,7 @@
       <c r="E3" s="85">
         <v>300</v>
       </c>
-      <c r="F3" s="135">
+      <c r="F3" s="128">
         <v>1</v>
       </c>
     </row>
@@ -11069,44 +11054,44 @@
   <sheetData>
     <row r="1" spans="1:14" ht="15.75" thickBot="1"/>
     <row r="2" spans="1:14" ht="15.75" thickBot="1">
-      <c r="B2" s="139" t="s">
+      <c r="B2" s="132" t="s">
         <v>257</v>
       </c>
-      <c r="C2" s="87" t="s">
+      <c r="C2" s="142" t="s">
+        <v>259</v>
+      </c>
+      <c r="D2" s="144" t="s">
+        <v>259</v>
+      </c>
+      <c r="E2" s="144" t="s">
+        <v>258</v>
+      </c>
+      <c r="F2" s="145" t="s">
         <v>260</v>
       </c>
-      <c r="D2" s="86" t="s">
-        <v>258</v>
-      </c>
-      <c r="E2" s="123" t="s">
-        <v>260</v>
-      </c>
-      <c r="F2" s="93" t="s">
-        <v>259</v>
-      </c>
-      <c r="G2" s="124"/>
+      <c r="G2" s="117"/>
     </row>
     <row r="3" spans="1:14">
-      <c r="B3" s="89" t="s">
+      <c r="B3" s="87" t="s">
         <v>253</v>
       </c>
-      <c r="C3" s="91">
-        <f>C4+C5*60+C6*3600+C7*3600*24</f>
-        <v>3600</v>
-      </c>
-      <c r="D3" s="92">
-        <f>C3+D4+D5*60+D6*3600+D7*3600*24</f>
-        <v>3720</v>
-      </c>
-      <c r="E3" s="92">
-        <f t="shared" ref="E3" si="0">D3+E4+E5*60+E6*3600+E7*3600*24</f>
-        <v>10920</v>
-      </c>
-      <c r="F3" s="94">
-        <f>E3+F4+F5*60+F6*3600+F7*3600*24</f>
-        <v>18120</v>
-      </c>
-      <c r="G3" s="96"/>
+      <c r="C3" s="89">
+        <f>IFERROR(C4+C5*60+C6*3600+C7*3600*24+B3,C4+C5*60+C6*3600+C7*3600*24)</f>
+        <v>32400</v>
+      </c>
+      <c r="D3" s="89">
+        <f t="shared" ref="D3:F3" si="0">IFERROR(D4+D5*60+D6*3600+D7*3600*24+C3,D4+D5*60+D6*3600+D7*3600*24)</f>
+        <v>32400</v>
+      </c>
+      <c r="E3" s="89">
+        <f t="shared" si="0"/>
+        <v>32400</v>
+      </c>
+      <c r="F3" s="89">
+        <f t="shared" si="0"/>
+        <v>32460</v>
+      </c>
+      <c r="G3" s="91"/>
       <c r="H3" s="81"/>
       <c r="I3" s="81"/>
       <c r="J3" s="81"/>
@@ -11116,924 +11101,918 @@
       <c r="N3" s="81"/>
     </row>
     <row r="4" spans="1:14">
-      <c r="B4" s="90" t="s">
+      <c r="B4" s="88" t="s">
         <v>256</v>
       </c>
-      <c r="C4" s="88"/>
+      <c r="C4" s="86"/>
       <c r="D4" s="84"/>
       <c r="E4" s="83"/>
-      <c r="F4" s="95"/>
-      <c r="G4" s="96"/>
+      <c r="F4" s="90"/>
+      <c r="G4" s="91"/>
     </row>
     <row r="5" spans="1:14">
-      <c r="B5" s="90" t="s">
+      <c r="B5" s="88" t="s">
         <v>255</v>
       </c>
-      <c r="C5" s="88"/>
-      <c r="D5" s="84">
-        <v>2</v>
-      </c>
+      <c r="C5" s="86"/>
+      <c r="D5" s="84"/>
       <c r="E5" s="83"/>
-      <c r="F5" s="95">
-        <v>0</v>
-      </c>
-      <c r="G5" s="96"/>
+      <c r="F5" s="90">
+        <v>1</v>
+      </c>
+      <c r="G5" s="91"/>
     </row>
     <row r="6" spans="1:14">
-      <c r="B6" s="90" t="s">
+      <c r="B6" s="88" t="s">
         <v>254</v>
       </c>
-      <c r="C6" s="88">
-        <v>1</v>
+      <c r="C6" s="143">
+        <v>9</v>
       </c>
       <c r="D6" s="84"/>
-      <c r="E6" s="83">
-        <v>2</v>
-      </c>
-      <c r="F6" s="95">
-        <v>2</v>
-      </c>
-      <c r="G6" s="96"/>
+      <c r="E6" s="83"/>
+      <c r="F6" s="90"/>
+      <c r="G6" s="91"/>
     </row>
     <row r="7" spans="1:14">
-      <c r="B7" s="118" t="s">
+      <c r="B7" s="112" t="s">
         <v>261</v>
       </c>
-      <c r="C7" s="119"/>
-      <c r="D7" s="120"/>
-      <c r="E7" s="121"/>
-      <c r="F7" s="122"/>
-      <c r="G7" s="96"/>
+      <c r="C7" s="113"/>
+      <c r="D7" s="114"/>
+      <c r="E7" s="115"/>
+      <c r="F7" s="116"/>
+      <c r="G7" s="91"/>
     </row>
     <row r="8" spans="1:14">
       <c r="A8" s="82">
         <v>1</v>
       </c>
-      <c r="B8" s="97" t="str">
+      <c r="B8" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A8+1)</f>
         <v>Frame 1, +X</v>
       </c>
-      <c r="C8" s="98">
+      <c r="C8" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A8+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D8" s="99">
+      <c r="D8" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A8+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E8" s="99">
+      <c r="E8" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A8+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F8" s="100">
+      <c r="F8" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A8+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G8" s="100"/>
-      <c r="H8" s="100"/>
-      <c r="I8" s="100"/>
-      <c r="J8" s="100"/>
-      <c r="K8" s="100"/>
+      <c r="G8" s="94"/>
+      <c r="H8" s="94"/>
+      <c r="I8" s="94"/>
+      <c r="J8" s="94"/>
+      <c r="K8" s="94"/>
     </row>
     <row r="9" spans="1:14">
       <c r="A9" s="82">
         <v>2</v>
       </c>
-      <c r="B9" s="97" t="str">
+      <c r="B9" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A9+1)</f>
         <v>Frame 2, -X</v>
       </c>
-      <c r="C9" s="98">
+      <c r="C9" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A9+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D9" s="99">
+      <c r="D9" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A9+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E9" s="99">
+      <c r="E9" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A9+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F9" s="100">
+      <c r="F9" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A9+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G9" s="100"/>
-      <c r="H9" s="100"/>
-      <c r="I9" s="100"/>
-      <c r="J9" s="100"/>
-      <c r="K9" s="100"/>
+      <c r="G9" s="94"/>
+      <c r="H9" s="94"/>
+      <c r="I9" s="94"/>
+      <c r="J9" s="94"/>
+      <c r="K9" s="94"/>
     </row>
     <row r="10" spans="1:14">
       <c r="A10" s="82">
         <v>3</v>
       </c>
-      <c r="B10" s="97" t="str">
+      <c r="B10" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A10+1)</f>
         <v>Beam -Y +Z</v>
       </c>
-      <c r="C10" s="98">
+      <c r="C10" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A10+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D10" s="99">
+      <c r="D10" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A10+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E10" s="99">
+      <c r="E10" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A10+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F10" s="100">
+      <c r="F10" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A10+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G10" s="100"/>
-      <c r="H10" s="100"/>
-      <c r="I10" s="100"/>
-      <c r="J10" s="100"/>
-      <c r="K10" s="100"/>
+      <c r="G10" s="94"/>
+      <c r="H10" s="94"/>
+      <c r="I10" s="94"/>
+      <c r="J10" s="94"/>
+      <c r="K10" s="94"/>
     </row>
     <row r="11" spans="1:14">
       <c r="A11" s="82">
         <v>4</v>
       </c>
-      <c r="B11" s="97" t="str">
+      <c r="B11" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A11+1)</f>
         <v>Beam +Y +Z</v>
       </c>
-      <c r="C11" s="98">
+      <c r="C11" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A11+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D11" s="99">
+      <c r="D11" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A11+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E11" s="99">
+      <c r="E11" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A11+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F11" s="100">
+      <c r="F11" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A11+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G11" s="100"/>
-      <c r="H11" s="100"/>
-      <c r="I11" s="100"/>
-      <c r="J11" s="100"/>
-      <c r="K11" s="100"/>
+      <c r="G11" s="94"/>
+      <c r="H11" s="94"/>
+      <c r="I11" s="94"/>
+      <c r="J11" s="94"/>
+      <c r="K11" s="94"/>
     </row>
     <row r="12" spans="1:14">
       <c r="A12" s="82">
         <v>5</v>
       </c>
-      <c r="B12" s="97" t="str">
+      <c r="B12" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A12+1)</f>
         <v>Beam +Y -Z</v>
       </c>
-      <c r="C12" s="98">
+      <c r="C12" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A12+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D12" s="99">
+      <c r="D12" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A12+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E12" s="99">
+      <c r="E12" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A12+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F12" s="100">
+      <c r="F12" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A12+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G12" s="100"/>
-      <c r="H12" s="100"/>
-      <c r="I12" s="100"/>
-      <c r="J12" s="100"/>
-      <c r="K12" s="100"/>
+      <c r="G12" s="94"/>
+      <c r="H12" s="94"/>
+      <c r="I12" s="94"/>
+      <c r="J12" s="94"/>
+      <c r="K12" s="94"/>
     </row>
     <row r="13" spans="1:14">
       <c r="A13" s="82">
         <v>6</v>
       </c>
-      <c r="B13" s="97" t="str">
+      <c r="B13" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A13+1)</f>
         <v>Beam -Y -Z</v>
       </c>
-      <c r="C13" s="98">
+      <c r="C13" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A13+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D13" s="99">
+      <c r="D13" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A13+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E13" s="99">
+      <c r="E13" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A13+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F13" s="100">
+      <c r="F13" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A13+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G13" s="100"/>
-      <c r="H13" s="100"/>
-      <c r="I13" s="100"/>
-      <c r="J13" s="100"/>
-      <c r="K13" s="100"/>
+      <c r="G13" s="94"/>
+      <c r="H13" s="94"/>
+      <c r="I13" s="94"/>
+      <c r="J13" s="94"/>
+      <c r="K13" s="94"/>
     </row>
     <row r="14" spans="1:14">
       <c r="A14" s="82">
         <v>7</v>
       </c>
-      <c r="B14" s="97" t="str">
+      <c r="B14" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A14+1)</f>
         <v xml:space="preserve">panel +Z, payload plate </v>
       </c>
-      <c r="C14" s="98">
+      <c r="C14" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A14+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D14" s="99">
+      <c r="D14" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A14+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E14" s="99">
+      <c r="E14" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A14+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F14" s="100">
+      <c r="F14" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A14+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G14" s="100"/>
-      <c r="H14" s="100"/>
-      <c r="I14" s="100"/>
-      <c r="J14" s="100"/>
-      <c r="K14" s="100"/>
+      <c r="G14" s="94"/>
+      <c r="H14" s="94"/>
+      <c r="I14" s="94"/>
+      <c r="J14" s="94"/>
+      <c r="K14" s="94"/>
     </row>
     <row r="15" spans="1:14">
       <c r="A15" s="82">
         <v>8</v>
       </c>
-      <c r="B15" s="97" t="str">
+      <c r="B15" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A15+1)</f>
         <v xml:space="preserve">LED 1 </v>
       </c>
-      <c r="C15" s="98">
+      <c r="C15" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A15+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="D15" s="99">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D15" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A15+1,FALSE)</f>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E15" s="93">
+        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A15+1,FALSE)</f>
         <v>200</v>
       </c>
-      <c r="E15" s="99">
-        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A15+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="F15" s="100">
+      <c r="F15" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A15+1,FALSE)</f>
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="G15" s="100"/>
-      <c r="H15" s="100"/>
-      <c r="I15" s="100"/>
-      <c r="J15" s="100"/>
-      <c r="K15" s="100"/>
+        <v>0</v>
+      </c>
+      <c r="G15" s="94"/>
+      <c r="H15" s="94"/>
+      <c r="I15" s="94"/>
+      <c r="J15" s="94"/>
+      <c r="K15" s="94"/>
     </row>
     <row r="16" spans="1:14">
       <c r="A16" s="82">
         <v>9</v>
       </c>
-      <c r="B16" s="97" t="str">
+      <c r="B16" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A16+1)</f>
         <v>LED 2</v>
       </c>
-      <c r="C16" s="98">
+      <c r="C16" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A16+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="D16" s="99">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D16" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A16+1,FALSE)</f>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E16" s="93">
+        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A16+1,FALSE)</f>
         <v>200</v>
       </c>
-      <c r="E16" s="99">
-        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A16+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="F16" s="100">
+      <c r="F16" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A16+1,FALSE)</f>
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="G16" s="100"/>
-      <c r="H16" s="100"/>
-      <c r="I16" s="100"/>
-      <c r="J16" s="100"/>
-      <c r="K16" s="100"/>
+        <v>0</v>
+      </c>
+      <c r="G16" s="94"/>
+      <c r="H16" s="94"/>
+      <c r="I16" s="94"/>
+      <c r="J16" s="94"/>
+      <c r="K16" s="94"/>
     </row>
     <row r="17" spans="1:11">
       <c r="A17" s="82">
         <v>10</v>
       </c>
-      <c r="B17" s="97" t="str">
+      <c r="B17" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A17+1)</f>
         <v>LED 3</v>
       </c>
-      <c r="C17" s="98">
+      <c r="C17" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A17+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="D17" s="99">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D17" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A17+1,FALSE)</f>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E17" s="93">
+        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A17+1,FALSE)</f>
         <v>200</v>
       </c>
-      <c r="E17" s="99">
-        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A17+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="F17" s="100">
+      <c r="F17" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A17+1,FALSE)</f>
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="G17" s="100"/>
-      <c r="H17" s="100"/>
-      <c r="I17" s="100"/>
-      <c r="J17" s="100"/>
-      <c r="K17" s="100"/>
+        <v>0</v>
+      </c>
+      <c r="G17" s="94"/>
+      <c r="H17" s="94"/>
+      <c r="I17" s="94"/>
+      <c r="J17" s="94"/>
+      <c r="K17" s="94"/>
     </row>
     <row r="18" spans="1:11">
       <c r="A18" s="82">
         <v>11</v>
       </c>
-      <c r="B18" s="97" t="str">
+      <c r="B18" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A18+1)</f>
         <v xml:space="preserve">LED 4 </v>
       </c>
-      <c r="C18" s="98">
+      <c r="C18" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A18+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="D18" s="99">
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="D18" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A18+1,FALSE)</f>
+        <v>5.0999999999999996</v>
+      </c>
+      <c r="E18" s="93">
+        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A18+1,FALSE)</f>
         <v>200</v>
       </c>
-      <c r="E18" s="99">
-        <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A18+1,FALSE)</f>
-        <v>0</v>
-      </c>
-      <c r="F18" s="100">
+      <c r="F18" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A18+1,FALSE)</f>
-        <v>5.0999999999999996</v>
-      </c>
-      <c r="G18" s="100"/>
-      <c r="H18" s="100"/>
-      <c r="I18" s="100"/>
-      <c r="J18" s="100"/>
-      <c r="K18" s="100"/>
+        <v>0</v>
+      </c>
+      <c r="G18" s="94"/>
+      <c r="H18" s="94"/>
+      <c r="I18" s="94"/>
+      <c r="J18" s="94"/>
+      <c r="K18" s="94"/>
     </row>
     <row r="19" spans="1:11">
       <c r="A19" s="82">
         <v>12</v>
       </c>
-      <c r="B19" s="97" t="str">
+      <c r="B19" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A19+1)</f>
         <v>Node 12, BMS</v>
       </c>
-      <c r="C19" s="98">
+      <c r="C19" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A19+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D19" s="99">
+      <c r="D19" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A19+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E19" s="99">
+      <c r="E19" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A19+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F19" s="100">
+      <c r="F19" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A19+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G19" s="100"/>
-      <c r="H19" s="100"/>
-      <c r="I19" s="100"/>
-      <c r="J19" s="100"/>
-      <c r="K19" s="100"/>
+      <c r="G19" s="94"/>
+      <c r="H19" s="94"/>
+      <c r="I19" s="94"/>
+      <c r="J19" s="94"/>
+      <c r="K19" s="94"/>
     </row>
     <row r="20" spans="1:11">
       <c r="A20" s="82">
         <v>13</v>
       </c>
-      <c r="B20" s="97" t="str">
+      <c r="B20" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A20+1)</f>
         <v>Node 13, Batteries Isolation</v>
       </c>
-      <c r="C20" s="98">
+      <c r="C20" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A20+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D20" s="99">
+      <c r="D20" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A20+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E20" s="99">
+      <c r="E20" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A20+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F20" s="100">
+      <c r="F20" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A20+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G20" s="100"/>
-      <c r="H20" s="100"/>
-      <c r="I20" s="100"/>
-      <c r="J20" s="100"/>
-      <c r="K20" s="100"/>
+      <c r="G20" s="94"/>
+      <c r="H20" s="94"/>
+      <c r="I20" s="94"/>
+      <c r="J20" s="94"/>
+      <c r="K20" s="94"/>
     </row>
     <row r="21" spans="1:11">
       <c r="A21" s="82">
         <v>14</v>
       </c>
-      <c r="B21" s="97" t="str">
+      <c r="B21" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A21+1)</f>
         <v>Node 14, LiFePo4 1</v>
       </c>
-      <c r="C21" s="98">
+      <c r="C21" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A21+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D21" s="99">
+      <c r="D21" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A21+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E21" s="99">
+      <c r="E21" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A21+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F21" s="100">
+      <c r="F21" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A21+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G21" s="100"/>
-      <c r="H21" s="100"/>
-      <c r="I21" s="100"/>
-      <c r="J21" s="100"/>
-      <c r="K21" s="100"/>
+      <c r="G21" s="94"/>
+      <c r="H21" s="94"/>
+      <c r="I21" s="94"/>
+      <c r="J21" s="94"/>
+      <c r="K21" s="94"/>
     </row>
     <row r="22" spans="1:11">
       <c r="A22" s="82">
         <v>15</v>
       </c>
-      <c r="B22" s="97" t="str">
+      <c r="B22" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A22+1)</f>
         <v>Node 15, LiFePo4 3</v>
       </c>
-      <c r="C22" s="98">
+      <c r="C22" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A22+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D22" s="99">
+      <c r="D22" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A22+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E22" s="99">
+      <c r="E22" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A22+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F22" s="100">
+      <c r="F22" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A22+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G22" s="100"/>
-      <c r="H22" s="100"/>
-      <c r="I22" s="100"/>
-      <c r="J22" s="100"/>
-      <c r="K22" s="100"/>
+      <c r="G22" s="94"/>
+      <c r="H22" s="94"/>
+      <c r="I22" s="94"/>
+      <c r="J22" s="94"/>
+      <c r="K22" s="94"/>
     </row>
     <row r="23" spans="1:11">
       <c r="A23" s="82">
         <v>16</v>
       </c>
-      <c r="B23" s="97" t="str">
+      <c r="B23" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A23+1)</f>
         <v>Node 16, LiFePo4 2</v>
       </c>
-      <c r="C23" s="98">
+      <c r="C23" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A23+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D23" s="99">
+      <c r="D23" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A23+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E23" s="99">
+      <c r="E23" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A23+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F23" s="100">
+      <c r="F23" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A23+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G23" s="100"/>
-      <c r="H23" s="100"/>
-      <c r="I23" s="100"/>
-      <c r="J23" s="100"/>
-      <c r="K23" s="100"/>
+      <c r="G23" s="94"/>
+      <c r="H23" s="94"/>
+      <c r="I23" s="94"/>
+      <c r="J23" s="94"/>
+      <c r="K23" s="94"/>
     </row>
     <row r="24" spans="1:11">
       <c r="A24" s="82">
         <v>17</v>
       </c>
-      <c r="B24" s="97" t="str">
+      <c r="B24" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A24+1)</f>
         <v>Node 17, LiFePo4 4</v>
       </c>
-      <c r="C24" s="98">
+      <c r="C24" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A24+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D24" s="99">
+      <c r="D24" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A24+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E24" s="99">
+      <c r="E24" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A24+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F24" s="100">
+      <c r="F24" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A24+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G24" s="100"/>
-      <c r="H24" s="100"/>
-      <c r="I24" s="100"/>
-      <c r="J24" s="100"/>
-      <c r="K24" s="100"/>
+      <c r="G24" s="94"/>
+      <c r="H24" s="94"/>
+      <c r="I24" s="94"/>
+      <c r="J24" s="94"/>
+      <c r="K24" s="94"/>
     </row>
     <row r="25" spans="1:11">
       <c r="A25" s="82">
         <v>18</v>
       </c>
-      <c r="B25" s="97" t="str">
+      <c r="B25" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A25+1)</f>
         <v>Node 18, Cell Litio 1</v>
       </c>
-      <c r="C25" s="98">
+      <c r="C25" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A25+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D25" s="99">
+      <c r="D25" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A25+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E25" s="99">
+      <c r="E25" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A25+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F25" s="100">
+      <c r="F25" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A25+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G25" s="100"/>
-      <c r="H25" s="100"/>
-      <c r="I25" s="100"/>
-      <c r="J25" s="100"/>
-      <c r="K25" s="100"/>
+      <c r="G25" s="94"/>
+      <c r="H25" s="94"/>
+      <c r="I25" s="94"/>
+      <c r="J25" s="94"/>
+      <c r="K25" s="94"/>
     </row>
     <row r="26" spans="1:11">
       <c r="A26" s="82">
         <v>19</v>
       </c>
-      <c r="B26" s="97" t="str">
+      <c r="B26" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A26+1)</f>
         <v>Node 19, Cell Litio 2</v>
       </c>
-      <c r="C26" s="98">
+      <c r="C26" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A26+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D26" s="99">
+      <c r="D26" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A26+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E26" s="99">
+      <c r="E26" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A26+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F26" s="100">
+      <c r="F26" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A26+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G26" s="100"/>
-      <c r="H26" s="100"/>
-      <c r="I26" s="100"/>
-      <c r="J26" s="100"/>
-      <c r="K26" s="100"/>
+      <c r="G26" s="94"/>
+      <c r="H26" s="94"/>
+      <c r="I26" s="94"/>
+      <c r="J26" s="94"/>
+      <c r="K26" s="94"/>
     </row>
     <row r="27" spans="1:11">
       <c r="A27" s="82">
         <v>20</v>
       </c>
-      <c r="B27" s="97" t="str">
+      <c r="B27" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A27+1)</f>
         <v>Node 20, LoMo</v>
       </c>
-      <c r="C27" s="98">
+      <c r="C27" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A27+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D27" s="99">
+      <c r="D27" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A27+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E27" s="99">
+      <c r="E27" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A27+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F27" s="100">
+      <c r="F27" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A27+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G27" s="100"/>
-      <c r="H27" s="100"/>
-      <c r="I27" s="100"/>
-      <c r="J27" s="100"/>
-      <c r="K27" s="100"/>
+      <c r="G27" s="94"/>
+      <c r="H27" s="94"/>
+      <c r="I27" s="94"/>
+      <c r="J27" s="94"/>
+      <c r="K27" s="94"/>
     </row>
     <row r="28" spans="1:11">
       <c r="A28" s="82">
         <v>21</v>
       </c>
-      <c r="B28" s="97" t="str">
+      <c r="B28" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A28+1)</f>
         <v>Node 21, Transceiver(Tx-Rx)</v>
       </c>
-      <c r="C28" s="98">
+      <c r="C28" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A28+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D28" s="99">
+      <c r="D28" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A28+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E28" s="99">
+      <c r="E28" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A28+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F28" s="100">
+      <c r="F28" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A28+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G28" s="100"/>
-      <c r="H28" s="100"/>
-      <c r="I28" s="100"/>
-      <c r="J28" s="100"/>
-      <c r="K28" s="100"/>
+      <c r="G28" s="94"/>
+      <c r="H28" s="94"/>
+      <c r="I28" s="94"/>
+      <c r="J28" s="94"/>
+      <c r="K28" s="94"/>
     </row>
     <row r="29" spans="1:11">
       <c r="A29" s="82">
         <v>22</v>
       </c>
-      <c r="B29" s="97" t="str">
+      <c r="B29" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A29+1)</f>
         <v>Node 22, Antena module</v>
       </c>
-      <c r="C29" s="98">
+      <c r="C29" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A29+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D29" s="99">
+      <c r="D29" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A29+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E29" s="99">
+      <c r="E29" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A29+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F29" s="100">
+      <c r="F29" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A29+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G29" s="100"/>
-      <c r="H29" s="100"/>
-      <c r="I29" s="100"/>
-      <c r="J29" s="100"/>
-      <c r="K29" s="100"/>
+      <c r="G29" s="94"/>
+      <c r="H29" s="94"/>
+      <c r="I29" s="94"/>
+      <c r="J29" s="94"/>
+      <c r="K29" s="94"/>
     </row>
     <row r="30" spans="1:11">
       <c r="A30" s="82">
         <v>23</v>
       </c>
-      <c r="B30" s="97" t="str">
+      <c r="B30" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A30+1)</f>
         <v>Node 23, OBC</v>
       </c>
-      <c r="C30" s="98">
+      <c r="C30" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A30+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D30" s="99">
+      <c r="D30" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A30+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E30" s="99">
+      <c r="E30" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A30+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F30" s="100">
+      <c r="F30" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A30+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G30" s="100"/>
-      <c r="H30" s="100"/>
-      <c r="I30" s="100"/>
-      <c r="J30" s="100"/>
-      <c r="K30" s="100"/>
+      <c r="G30" s="94"/>
+      <c r="H30" s="94"/>
+      <c r="I30" s="94"/>
+      <c r="J30" s="94"/>
+      <c r="K30" s="94"/>
     </row>
     <row r="31" spans="1:11">
       <c r="A31" s="82">
         <v>24</v>
       </c>
-      <c r="B31" s="97" t="str">
+      <c r="B31" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A31+1)</f>
         <v>Node 24, Solar Panel (Y)</v>
       </c>
-      <c r="C31" s="98">
+      <c r="C31" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A31+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D31" s="99">
+      <c r="D31" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A31+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E31" s="99">
+      <c r="E31" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A31+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F31" s="100">
+      <c r="F31" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A31+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G31" s="100"/>
-      <c r="H31" s="100"/>
-      <c r="I31" s="100"/>
-      <c r="J31" s="100"/>
-      <c r="K31" s="100"/>
+      <c r="G31" s="94"/>
+      <c r="H31" s="94"/>
+      <c r="I31" s="94"/>
+      <c r="J31" s="94"/>
+      <c r="K31" s="94"/>
     </row>
     <row r="32" spans="1:11">
       <c r="A32" s="82">
         <v>25</v>
       </c>
-      <c r="B32" s="97" t="str">
+      <c r="B32" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A32+1)</f>
         <v>Node 25, Solar Panel (-Y)</v>
       </c>
-      <c r="C32" s="98">
+      <c r="C32" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A32+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D32" s="99">
+      <c r="D32" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A32+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E32" s="99">
+      <c r="E32" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A32+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F32" s="100">
+      <c r="F32" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A32+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G32" s="100"/>
-      <c r="H32" s="100"/>
-      <c r="I32" s="100"/>
-      <c r="J32" s="100"/>
-      <c r="K32" s="100"/>
+      <c r="G32" s="94"/>
+      <c r="H32" s="94"/>
+      <c r="I32" s="94"/>
+      <c r="J32" s="94"/>
+      <c r="K32" s="94"/>
     </row>
     <row r="33" spans="1:11">
       <c r="A33" s="82">
         <v>26</v>
       </c>
-      <c r="B33" s="97" t="str">
+      <c r="B33" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A33+1)</f>
         <v>Node 26, Solar Panel (X)</v>
       </c>
-      <c r="C33" s="98">
+      <c r="C33" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A33+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D33" s="99">
+      <c r="D33" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A33+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E33" s="99">
+      <c r="E33" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A33+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F33" s="100">
+      <c r="F33" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A33+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G33" s="100"/>
-      <c r="H33" s="100"/>
-      <c r="I33" s="100"/>
-      <c r="J33" s="100"/>
-      <c r="K33" s="100"/>
+      <c r="G33" s="94"/>
+      <c r="H33" s="94"/>
+      <c r="I33" s="94"/>
+      <c r="J33" s="94"/>
+      <c r="K33" s="94"/>
     </row>
     <row r="34" spans="1:11">
       <c r="A34" s="82">
         <v>27</v>
       </c>
-      <c r="B34" s="97" t="str">
+      <c r="B34" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A34+1)</f>
         <v>Node 27, Solar Panel (-X)RBF</v>
       </c>
-      <c r="C34" s="98">
+      <c r="C34" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A34+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D34" s="99">
+      <c r="D34" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A34+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E34" s="99">
+      <c r="E34" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A34+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F34" s="100">
+      <c r="F34" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A34+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G34" s="100"/>
-      <c r="H34" s="100"/>
-      <c r="I34" s="100"/>
-      <c r="J34" s="100"/>
-      <c r="K34" s="100"/>
+      <c r="G34" s="94"/>
+      <c r="H34" s="94"/>
+      <c r="I34" s="94"/>
+      <c r="J34" s="94"/>
+      <c r="K34" s="94"/>
     </row>
     <row r="35" spans="1:11">
       <c r="A35" s="82">
         <v>28</v>
       </c>
-      <c r="B35" s="97" t="str">
+      <c r="B35" s="92" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A35+1)</f>
         <v>Node 28, Solar Panel (-Z(antenna))</v>
       </c>
-      <c r="C35" s="98">
+      <c r="C35" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A35+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D35" s="99">
+      <c r="D35" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A35+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E35" s="99">
+      <c r="E35" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A35+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F35" s="100">
+      <c r="F35" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A35+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G35" s="100"/>
-      <c r="H35" s="100"/>
-      <c r="I35" s="100"/>
-      <c r="J35" s="100"/>
-      <c r="K35" s="100"/>
+      <c r="G35" s="94"/>
+      <c r="H35" s="94"/>
+      <c r="I35" s="94"/>
+      <c r="J35" s="94"/>
+      <c r="K35" s="94"/>
     </row>
     <row r="36" spans="1:11" ht="15.75" thickBot="1">
       <c r="A36" s="82">
         <v>29</v>
       </c>
-      <c r="B36" s="101" t="str">
+      <c r="B36" s="95" t="str">
         <f>HLOOKUP(B$2,Modes!$B$2:$E$31,$A36+1)</f>
         <v>Node 29, EPS de alta</v>
       </c>
-      <c r="C36" s="98">
+      <c r="C36" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A36+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="D36" s="99">
+      <c r="D36" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A36+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="E36" s="99">
+      <c r="E36" s="93">
         <f>HLOOKUP(E$2,Modes!$B$2:$O$31,$A36+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="F36" s="100">
+      <c r="F36" s="93">
         <f>HLOOKUP(F$2,Modes!$B$2:$O$31,$A36+1,FALSE)</f>
         <v>0</v>
       </c>
-      <c r="G36" s="100"/>
-      <c r="H36" s="100"/>
-      <c r="I36" s="100"/>
-      <c r="J36" s="100"/>
-      <c r="K36" s="100"/>
+      <c r="G36" s="94"/>
+      <c r="H36" s="94"/>
+      <c r="I36" s="94"/>
+      <c r="J36" s="94"/>
+      <c r="K36" s="94"/>
     </row>
     <row r="37" spans="1:11">
       <c r="B37" s="80"/>
@@ -12053,58 +12032,58 @@
   <sheetData>
     <row r="1" spans="2:15" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:15" ht="15.75" thickBot="1">
-      <c r="B2" s="140" t="s">
+      <c r="B2" s="133" t="s">
         <v>257</v>
       </c>
-      <c r="C2" s="125" t="s">
+      <c r="C2" s="118" t="s">
         <v>260</v>
       </c>
-      <c r="D2" s="126" t="s">
+      <c r="D2" s="119" t="s">
         <v>258</v>
       </c>
-      <c r="E2" s="126" t="s">
+      <c r="E2" s="119" t="s">
         <v>259</v>
       </c>
-      <c r="F2" s="127"/>
-      <c r="G2" s="127"/>
-      <c r="H2" s="127"/>
-      <c r="I2" s="127"/>
-      <c r="J2" s="127"/>
-      <c r="K2" s="127"/>
-      <c r="L2" s="127"/>
-      <c r="M2" s="127"/>
-      <c r="N2" s="127"/>
-      <c r="O2" s="128"/>
+      <c r="F2" s="120"/>
+      <c r="G2" s="120"/>
+      <c r="H2" s="120"/>
+      <c r="I2" s="120"/>
+      <c r="J2" s="120"/>
+      <c r="K2" s="120"/>
+      <c r="L2" s="120"/>
+      <c r="M2" s="120"/>
+      <c r="N2" s="120"/>
+      <c r="O2" s="121"/>
     </row>
     <row r="3" spans="2:15">
-      <c r="B3" s="141" t="s">
+      <c r="B3" s="134" t="s">
         <v>214</v>
       </c>
-      <c r="C3" s="129">
-        <v>0</v>
-      </c>
-      <c r="D3" s="130">
-        <v>0</v>
-      </c>
-      <c r="E3" s="130">
-        <v>0</v>
-      </c>
-      <c r="F3" s="130"/>
-      <c r="G3" s="130"/>
-      <c r="H3" s="130"/>
-      <c r="I3" s="130"/>
-      <c r="J3" s="130"/>
-      <c r="K3" s="130"/>
-      <c r="L3" s="130"/>
-      <c r="M3" s="130"/>
-      <c r="N3" s="130"/>
-      <c r="O3" s="131"/>
+      <c r="C3" s="122">
+        <v>0</v>
+      </c>
+      <c r="D3" s="123">
+        <v>0</v>
+      </c>
+      <c r="E3" s="123">
+        <v>0</v>
+      </c>
+      <c r="F3" s="123"/>
+      <c r="G3" s="123"/>
+      <c r="H3" s="123"/>
+      <c r="I3" s="123"/>
+      <c r="J3" s="123"/>
+      <c r="K3" s="123"/>
+      <c r="L3" s="123"/>
+      <c r="M3" s="123"/>
+      <c r="N3" s="123"/>
+      <c r="O3" s="124"/>
     </row>
     <row r="4" spans="2:15">
-      <c r="B4" s="142" t="s">
+      <c r="B4" s="135" t="s">
         <v>215</v>
       </c>
-      <c r="C4" s="132">
+      <c r="C4" s="125">
         <v>0</v>
       </c>
       <c r="D4" s="84">
@@ -12122,13 +12101,13 @@
       <c r="L4" s="84"/>
       <c r="M4" s="84"/>
       <c r="N4" s="84"/>
-      <c r="O4" s="133"/>
+      <c r="O4" s="126"/>
     </row>
     <row r="5" spans="2:15">
-      <c r="B5" s="142" t="s">
+      <c r="B5" s="135" t="s">
         <v>216</v>
       </c>
-      <c r="C5" s="132">
+      <c r="C5" s="125">
         <v>0</v>
       </c>
       <c r="D5" s="84">
@@ -12146,13 +12125,13 @@
       <c r="L5" s="84"/>
       <c r="M5" s="84"/>
       <c r="N5" s="84"/>
-      <c r="O5" s="133"/>
+      <c r="O5" s="126"/>
     </row>
     <row r="6" spans="2:15">
-      <c r="B6" s="142" t="s">
+      <c r="B6" s="135" t="s">
         <v>217</v>
       </c>
-      <c r="C6" s="132">
+      <c r="C6" s="125">
         <v>0</v>
       </c>
       <c r="D6" s="84">
@@ -12170,13 +12149,13 @@
       <c r="L6" s="84"/>
       <c r="M6" s="84"/>
       <c r="N6" s="84"/>
-      <c r="O6" s="133"/>
+      <c r="O6" s="126"/>
     </row>
     <row r="7" spans="2:15">
-      <c r="B7" s="142" t="s">
+      <c r="B7" s="135" t="s">
         <v>218</v>
       </c>
-      <c r="C7" s="132">
+      <c r="C7" s="125">
         <v>0</v>
       </c>
       <c r="D7" s="84">
@@ -12194,13 +12173,13 @@
       <c r="L7" s="84"/>
       <c r="M7" s="84"/>
       <c r="N7" s="84"/>
-      <c r="O7" s="133"/>
+      <c r="O7" s="126"/>
     </row>
     <row r="8" spans="2:15">
-      <c r="B8" s="142" t="s">
+      <c r="B8" s="135" t="s">
         <v>219</v>
       </c>
-      <c r="C8" s="132">
+      <c r="C8" s="125">
         <v>0</v>
       </c>
       <c r="D8" s="84">
@@ -12218,13 +12197,13 @@
       <c r="L8" s="84"/>
       <c r="M8" s="84"/>
       <c r="N8" s="84"/>
-      <c r="O8" s="133"/>
+      <c r="O8" s="126"/>
     </row>
     <row r="9" spans="2:15">
-      <c r="B9" s="142" t="s">
+      <c r="B9" s="135" t="s">
         <v>220</v>
       </c>
-      <c r="C9" s="132">
+      <c r="C9" s="125">
         <v>0</v>
       </c>
       <c r="D9" s="84">
@@ -12242,13 +12221,13 @@
       <c r="L9" s="84"/>
       <c r="M9" s="84"/>
       <c r="N9" s="84"/>
-      <c r="O9" s="133"/>
+      <c r="O9" s="126"/>
     </row>
     <row r="10" spans="2:15">
-      <c r="B10" s="142" t="s">
+      <c r="B10" s="135" t="s">
         <v>221</v>
       </c>
-      <c r="C10" s="132">
+      <c r="C10" s="125">
         <v>0</v>
       </c>
       <c r="D10" s="84">
@@ -12266,13 +12245,13 @@
       <c r="L10" s="84"/>
       <c r="M10" s="84"/>
       <c r="N10" s="84"/>
-      <c r="O10" s="133"/>
+      <c r="O10" s="126"/>
     </row>
     <row r="11" spans="2:15">
-      <c r="B11" s="142" t="s">
+      <c r="B11" s="135" t="s">
         <v>222</v>
       </c>
-      <c r="C11" s="132">
+      <c r="C11" s="125">
         <v>0</v>
       </c>
       <c r="D11" s="84">
@@ -12290,13 +12269,13 @@
       <c r="L11" s="84"/>
       <c r="M11" s="84"/>
       <c r="N11" s="84"/>
-      <c r="O11" s="133"/>
+      <c r="O11" s="126"/>
     </row>
     <row r="12" spans="2:15">
-      <c r="B12" s="142" t="s">
+      <c r="B12" s="135" t="s">
         <v>223</v>
       </c>
-      <c r="C12" s="132">
+      <c r="C12" s="125">
         <v>0</v>
       </c>
       <c r="D12" s="84">
@@ -12314,13 +12293,13 @@
       <c r="L12" s="84"/>
       <c r="M12" s="84"/>
       <c r="N12" s="84"/>
-      <c r="O12" s="133"/>
+      <c r="O12" s="126"/>
     </row>
     <row r="13" spans="2:15">
-      <c r="B13" s="142" t="s">
+      <c r="B13" s="135" t="s">
         <v>224</v>
       </c>
-      <c r="C13" s="132">
+      <c r="C13" s="125">
         <v>0</v>
       </c>
       <c r="D13" s="84">
@@ -12338,13 +12317,13 @@
       <c r="L13" s="84"/>
       <c r="M13" s="84"/>
       <c r="N13" s="84"/>
-      <c r="O13" s="133"/>
+      <c r="O13" s="126"/>
     </row>
     <row r="14" spans="2:15">
-      <c r="B14" s="142" t="s">
+      <c r="B14" s="135" t="s">
         <v>225</v>
       </c>
-      <c r="C14" s="132">
+      <c r="C14" s="125">
         <v>0</v>
       </c>
       <c r="D14" s="84">
@@ -12362,13 +12341,13 @@
       <c r="L14" s="84"/>
       <c r="M14" s="84"/>
       <c r="N14" s="84"/>
-      <c r="O14" s="133"/>
+      <c r="O14" s="126"/>
     </row>
     <row r="15" spans="2:15">
-      <c r="B15" s="142" t="s">
+      <c r="B15" s="135" t="s">
         <v>226</v>
       </c>
-      <c r="C15" s="132">
+      <c r="C15" s="125">
         <v>0</v>
       </c>
       <c r="D15" s="84">
@@ -12386,13 +12365,13 @@
       <c r="L15" s="84"/>
       <c r="M15" s="84"/>
       <c r="N15" s="84"/>
-      <c r="O15" s="133"/>
+      <c r="O15" s="126"/>
     </row>
     <row r="16" spans="2:15">
-      <c r="B16" s="142" t="s">
+      <c r="B16" s="135" t="s">
         <v>227</v>
       </c>
-      <c r="C16" s="132">
+      <c r="C16" s="125">
         <v>0</v>
       </c>
       <c r="D16" s="84">
@@ -12410,13 +12389,13 @@
       <c r="L16" s="84"/>
       <c r="M16" s="84"/>
       <c r="N16" s="84"/>
-      <c r="O16" s="133"/>
+      <c r="O16" s="126"/>
     </row>
     <row r="17" spans="2:15">
-      <c r="B17" s="142" t="s">
+      <c r="B17" s="135" t="s">
         <v>228</v>
       </c>
-      <c r="C17" s="132">
+      <c r="C17" s="125">
         <v>0</v>
       </c>
       <c r="D17" s="84">
@@ -12434,13 +12413,13 @@
       <c r="L17" s="84"/>
       <c r="M17" s="84"/>
       <c r="N17" s="84"/>
-      <c r="O17" s="133"/>
+      <c r="O17" s="126"/>
     </row>
     <row r="18" spans="2:15">
-      <c r="B18" s="142" t="s">
+      <c r="B18" s="135" t="s">
         <v>229</v>
       </c>
-      <c r="C18" s="132">
+      <c r="C18" s="125">
         <v>0</v>
       </c>
       <c r="D18" s="84">
@@ -12458,13 +12437,13 @@
       <c r="L18" s="84"/>
       <c r="M18" s="84"/>
       <c r="N18" s="84"/>
-      <c r="O18" s="133"/>
+      <c r="O18" s="126"/>
     </row>
     <row r="19" spans="2:15">
-      <c r="B19" s="142" t="s">
+      <c r="B19" s="135" t="s">
         <v>230</v>
       </c>
-      <c r="C19" s="132">
+      <c r="C19" s="125">
         <v>0</v>
       </c>
       <c r="D19" s="84">
@@ -12482,13 +12461,13 @@
       <c r="L19" s="84"/>
       <c r="M19" s="84"/>
       <c r="N19" s="84"/>
-      <c r="O19" s="133"/>
+      <c r="O19" s="126"/>
     </row>
     <row r="20" spans="2:15">
-      <c r="B20" s="142" t="s">
+      <c r="B20" s="135" t="s">
         <v>231</v>
       </c>
-      <c r="C20" s="132">
+      <c r="C20" s="125">
         <v>0</v>
       </c>
       <c r="D20" s="84">
@@ -12506,13 +12485,13 @@
       <c r="L20" s="84"/>
       <c r="M20" s="84"/>
       <c r="N20" s="84"/>
-      <c r="O20" s="133"/>
+      <c r="O20" s="126"/>
     </row>
     <row r="21" spans="2:15">
-      <c r="B21" s="142" t="s">
+      <c r="B21" s="135" t="s">
         <v>232</v>
       </c>
-      <c r="C21" s="132">
+      <c r="C21" s="125">
         <v>0</v>
       </c>
       <c r="D21" s="84">
@@ -12530,13 +12509,13 @@
       <c r="L21" s="84"/>
       <c r="M21" s="84"/>
       <c r="N21" s="84"/>
-      <c r="O21" s="133"/>
+      <c r="O21" s="126"/>
     </row>
     <row r="22" spans="2:15">
-      <c r="B22" s="142" t="s">
+      <c r="B22" s="135" t="s">
         <v>233</v>
       </c>
-      <c r="C22" s="132">
+      <c r="C22" s="125">
         <v>0</v>
       </c>
       <c r="D22" s="84">
@@ -12554,13 +12533,13 @@
       <c r="L22" s="84"/>
       <c r="M22" s="84"/>
       <c r="N22" s="84"/>
-      <c r="O22" s="133"/>
+      <c r="O22" s="126"/>
     </row>
     <row r="23" spans="2:15">
-      <c r="B23" s="142" t="s">
+      <c r="B23" s="135" t="s">
         <v>234</v>
       </c>
-      <c r="C23" s="132">
+      <c r="C23" s="125">
         <v>0</v>
       </c>
       <c r="D23" s="84">
@@ -12578,13 +12557,13 @@
       <c r="L23" s="84"/>
       <c r="M23" s="84"/>
       <c r="N23" s="84"/>
-      <c r="O23" s="133"/>
+      <c r="O23" s="126"/>
     </row>
     <row r="24" spans="2:15">
-      <c r="B24" s="142" t="s">
+      <c r="B24" s="135" t="s">
         <v>235</v>
       </c>
-      <c r="C24" s="132">
+      <c r="C24" s="125">
         <v>0</v>
       </c>
       <c r="D24" s="84">
@@ -12602,13 +12581,13 @@
       <c r="L24" s="84"/>
       <c r="M24" s="84"/>
       <c r="N24" s="84"/>
-      <c r="O24" s="133"/>
+      <c r="O24" s="126"/>
     </row>
     <row r="25" spans="2:15">
-      <c r="B25" s="142" t="s">
+      <c r="B25" s="135" t="s">
         <v>236</v>
       </c>
-      <c r="C25" s="132">
+      <c r="C25" s="125">
         <v>0</v>
       </c>
       <c r="D25" s="84">
@@ -12626,13 +12605,13 @@
       <c r="L25" s="84"/>
       <c r="M25" s="84"/>
       <c r="N25" s="84"/>
-      <c r="O25" s="133"/>
+      <c r="O25" s="126"/>
     </row>
     <row r="26" spans="2:15">
-      <c r="B26" s="142" t="s">
+      <c r="B26" s="135" t="s">
         <v>237</v>
       </c>
-      <c r="C26" s="132">
+      <c r="C26" s="125">
         <v>0</v>
       </c>
       <c r="D26" s="84">
@@ -12650,13 +12629,13 @@
       <c r="L26" s="84"/>
       <c r="M26" s="84"/>
       <c r="N26" s="84"/>
-      <c r="O26" s="133"/>
+      <c r="O26" s="126"/>
     </row>
     <row r="27" spans="2:15">
-      <c r="B27" s="142" t="s">
+      <c r="B27" s="135" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="132">
+      <c r="C27" s="125">
         <v>0</v>
       </c>
       <c r="D27" s="84">
@@ -12674,13 +12653,13 @@
       <c r="L27" s="84"/>
       <c r="M27" s="84"/>
       <c r="N27" s="84"/>
-      <c r="O27" s="133"/>
+      <c r="O27" s="126"/>
     </row>
     <row r="28" spans="2:15">
-      <c r="B28" s="142" t="s">
+      <c r="B28" s="135" t="s">
         <v>239</v>
       </c>
-      <c r="C28" s="132">
+      <c r="C28" s="125">
         <v>0</v>
       </c>
       <c r="D28" s="84">
@@ -12698,13 +12677,13 @@
       <c r="L28" s="84"/>
       <c r="M28" s="84"/>
       <c r="N28" s="84"/>
-      <c r="O28" s="133"/>
+      <c r="O28" s="126"/>
     </row>
     <row r="29" spans="2:15">
-      <c r="B29" s="142" t="s">
+      <c r="B29" s="135" t="s">
         <v>240</v>
       </c>
-      <c r="C29" s="132">
+      <c r="C29" s="125">
         <v>0</v>
       </c>
       <c r="D29" s="84">
@@ -12722,13 +12701,13 @@
       <c r="L29" s="84"/>
       <c r="M29" s="84"/>
       <c r="N29" s="84"/>
-      <c r="O29" s="133"/>
+      <c r="O29" s="126"/>
     </row>
     <row r="30" spans="2:15">
-      <c r="B30" s="142" t="s">
+      <c r="B30" s="135" t="s">
         <v>241</v>
       </c>
-      <c r="C30" s="132">
+      <c r="C30" s="125">
         <v>0</v>
       </c>
       <c r="D30" s="84">
@@ -12746,47 +12725,47 @@
       <c r="L30" s="84"/>
       <c r="M30" s="84"/>
       <c r="N30" s="84"/>
-      <c r="O30" s="133"/>
+      <c r="O30" s="126"/>
     </row>
     <row r="31" spans="2:15">
-      <c r="B31" s="143" t="s">
+      <c r="B31" s="136" t="s">
         <v>242</v>
       </c>
-      <c r="C31" s="136">
-        <v>0</v>
-      </c>
-      <c r="D31" s="120">
-        <v>0</v>
-      </c>
-      <c r="E31" s="120">
-        <v>0</v>
-      </c>
-      <c r="F31" s="120"/>
-      <c r="G31" s="120"/>
-      <c r="H31" s="120"/>
-      <c r="I31" s="120"/>
-      <c r="J31" s="120"/>
-      <c r="K31" s="120"/>
-      <c r="L31" s="120"/>
-      <c r="M31" s="120"/>
-      <c r="N31" s="120"/>
-      <c r="O31" s="137"/>
+      <c r="C31" s="129">
+        <v>0</v>
+      </c>
+      <c r="D31" s="114">
+        <v>0</v>
+      </c>
+      <c r="E31" s="114">
+        <v>0</v>
+      </c>
+      <c r="F31" s="114"/>
+      <c r="G31" s="114"/>
+      <c r="H31" s="114"/>
+      <c r="I31" s="114"/>
+      <c r="J31" s="114"/>
+      <c r="K31" s="114"/>
+      <c r="L31" s="114"/>
+      <c r="M31" s="114"/>
+      <c r="N31" s="114"/>
+      <c r="O31" s="130"/>
     </row>
     <row r="32" spans="2:15">
-      <c r="B32" s="96"/>
-      <c r="C32" s="96"/>
-      <c r="D32" s="96"/>
-      <c r="E32" s="96"/>
-      <c r="F32" s="96"/>
-      <c r="G32" s="96"/>
-      <c r="H32" s="96"/>
-      <c r="I32" s="96"/>
-      <c r="J32" s="96"/>
-      <c r="K32" s="96"/>
-      <c r="L32" s="96"/>
-      <c r="M32" s="96"/>
-      <c r="N32" s="96"/>
-      <c r="O32" s="96"/>
+      <c r="B32" s="91"/>
+      <c r="C32" s="91"/>
+      <c r="D32" s="91"/>
+      <c r="E32" s="91"/>
+      <c r="F32" s="91"/>
+      <c r="G32" s="91"/>
+      <c r="H32" s="91"/>
+      <c r="I32" s="91"/>
+      <c r="J32" s="91"/>
+      <c r="K32" s="91"/>
+      <c r="L32" s="91"/>
+      <c r="M32" s="91"/>
+      <c r="N32" s="91"/>
+      <c r="O32" s="91"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -12812,922 +12791,922 @@
   <sheetData>
     <row r="1" spans="2:13" ht="15.75" thickBot="1"/>
     <row r="2" spans="2:13" ht="46.5" customHeight="1" thickBot="1">
-      <c r="B2" s="111" t="s">
+      <c r="B2" s="105" t="s">
         <v>252</v>
       </c>
-      <c r="C2" s="112" t="s">
+      <c r="C2" s="106" t="s">
         <v>245</v>
       </c>
-      <c r="D2" s="113" t="s">
+      <c r="D2" s="107" t="s">
         <v>246</v>
       </c>
-      <c r="E2" s="113" t="s">
+      <c r="E2" s="107" t="s">
         <v>248</v>
       </c>
-      <c r="F2" s="113" t="s">
+      <c r="F2" s="107" t="s">
         <v>247</v>
       </c>
-      <c r="G2" s="113" t="s">
+      <c r="G2" s="107" t="s">
         <v>243</v>
       </c>
-      <c r="H2" s="113" t="s">
+      <c r="H2" s="107" t="s">
         <v>244</v>
       </c>
-      <c r="I2" s="113" t="s">
+      <c r="I2" s="107" t="s">
         <v>249</v>
       </c>
-      <c r="J2" s="113" t="s">
+      <c r="J2" s="107" t="s">
         <v>250</v>
       </c>
-      <c r="K2" s="113" t="s">
+      <c r="K2" s="107" t="s">
         <v>251</v>
       </c>
-      <c r="L2" s="138" t="s">
+      <c r="L2" s="131" t="s">
         <v>262</v>
       </c>
-      <c r="M2" s="114" t="s">
+      <c r="M2" s="108" t="s">
         <v>213</v>
       </c>
     </row>
     <row r="3" spans="2:13">
-      <c r="B3" s="115" t="s">
+      <c r="B3" s="109" t="s">
         <v>214</v>
       </c>
-      <c r="C3" s="108">
+      <c r="C3" s="102">
         <v>4.0280000000000003E-2</v>
       </c>
-      <c r="D3" s="106">
+      <c r="D3" s="100">
         <v>800</v>
       </c>
-      <c r="E3" s="106"/>
-      <c r="F3" s="106">
+      <c r="E3" s="100"/>
+      <c r="F3" s="100">
         <v>5.1999999999999998E-3</v>
       </c>
-      <c r="G3" s="106">
+      <c r="G3" s="100">
         <v>0.8</v>
       </c>
-      <c r="H3" s="106">
+      <c r="H3" s="100">
         <v>0.8</v>
       </c>
-      <c r="I3" s="106">
+      <c r="I3" s="100">
         <v>1</v>
       </c>
-      <c r="J3" s="106">
-        <v>0</v>
-      </c>
-      <c r="K3" s="106">
-        <v>0</v>
-      </c>
-      <c r="L3" s="106">
+      <c r="J3" s="100">
+        <v>0</v>
+      </c>
+      <c r="K3" s="100">
+        <v>0</v>
+      </c>
+      <c r="L3" s="100">
         <v>1</v>
       </c>
-      <c r="M3" s="107"/>
+      <c r="M3" s="101"/>
     </row>
     <row r="4" spans="2:13">
-      <c r="B4" s="116" t="s">
+      <c r="B4" s="110" t="s">
         <v>215</v>
       </c>
-      <c r="C4" s="109">
+      <c r="C4" s="103">
         <v>4.0280000000000003E-2</v>
       </c>
-      <c r="D4" s="102">
+      <c r="D4" s="96">
         <v>800</v>
       </c>
-      <c r="E4" s="102"/>
-      <c r="F4" s="102">
+      <c r="E4" s="96"/>
+      <c r="F4" s="96">
         <v>5.1999999999999998E-3</v>
       </c>
-      <c r="G4" s="102">
+      <c r="G4" s="96">
         <v>0.8</v>
       </c>
-      <c r="H4" s="102">
+      <c r="H4" s="96">
         <v>0.8</v>
       </c>
-      <c r="I4" s="102">
+      <c r="I4" s="96">
         <v>-1</v>
       </c>
-      <c r="J4" s="102">
-        <v>0</v>
-      </c>
-      <c r="K4" s="102">
-        <v>0</v>
-      </c>
-      <c r="L4" s="102">
+      <c r="J4" s="96">
+        <v>0</v>
+      </c>
+      <c r="K4" s="96">
+        <v>0</v>
+      </c>
+      <c r="L4" s="96">
         <v>1</v>
       </c>
-      <c r="M4" s="104"/>
+      <c r="M4" s="98"/>
     </row>
     <row r="5" spans="2:13">
-      <c r="B5" s="116" t="s">
+      <c r="B5" s="110" t="s">
         <v>216</v>
       </c>
-      <c r="C5" s="109">
+      <c r="C5" s="103">
         <v>7.2909999999999997E-3</v>
       </c>
-      <c r="D5" s="102">
+      <c r="D5" s="96">
         <v>800</v>
       </c>
-      <c r="E5" s="102"/>
-      <c r="F5" s="102">
+      <c r="E5" s="96"/>
+      <c r="F5" s="96">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="G5" s="102">
+      <c r="G5" s="96">
         <v>0.8</v>
       </c>
-      <c r="H5" s="102">
+      <c r="H5" s="96">
         <v>0.8</v>
       </c>
-      <c r="I5" s="102">
-        <v>0</v>
-      </c>
-      <c r="J5" s="102">
+      <c r="I5" s="96">
+        <v>0</v>
+      </c>
+      <c r="J5" s="96">
         <v>-1</v>
       </c>
-      <c r="K5" s="102">
+      <c r="K5" s="96">
         <v>1</v>
       </c>
-      <c r="L5" s="102">
+      <c r="L5" s="96">
         <v>1</v>
       </c>
-      <c r="M5" s="104"/>
+      <c r="M5" s="98"/>
     </row>
     <row r="6" spans="2:13">
-      <c r="B6" s="116" t="s">
+      <c r="B6" s="110" t="s">
         <v>217</v>
       </c>
-      <c r="C6" s="109">
+      <c r="C6" s="103">
         <v>7.2909999999999997E-3</v>
       </c>
-      <c r="D6" s="102">
+      <c r="D6" s="96">
         <v>800</v>
       </c>
-      <c r="E6" s="102"/>
-      <c r="F6" s="102">
+      <c r="E6" s="96"/>
+      <c r="F6" s="96">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="G6" s="102">
+      <c r="G6" s="96">
         <v>0.8</v>
       </c>
-      <c r="H6" s="102">
+      <c r="H6" s="96">
         <v>0.8</v>
       </c>
-      <c r="I6" s="102">
-        <v>0</v>
-      </c>
-      <c r="J6" s="102">
+      <c r="I6" s="96">
+        <v>0</v>
+      </c>
+      <c r="J6" s="96">
         <v>1</v>
       </c>
-      <c r="K6" s="102">
+      <c r="K6" s="96">
         <v>1</v>
       </c>
-      <c r="L6" s="102">
+      <c r="L6" s="96">
         <v>1</v>
       </c>
-      <c r="M6" s="104"/>
+      <c r="M6" s="98"/>
     </row>
     <row r="7" spans="2:13">
-      <c r="B7" s="116" t="s">
+      <c r="B7" s="110" t="s">
         <v>218</v>
       </c>
-      <c r="C7" s="109">
+      <c r="C7" s="103">
         <v>6.4250000000000002E-3</v>
       </c>
-      <c r="D7" s="102">
+      <c r="D7" s="96">
         <v>800</v>
       </c>
-      <c r="E7" s="102"/>
-      <c r="F7" s="102">
+      <c r="E7" s="96"/>
+      <c r="F7" s="96">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="G7" s="102">
+      <c r="G7" s="96">
         <v>0.8</v>
       </c>
-      <c r="H7" s="102">
+      <c r="H7" s="96">
         <v>0.8</v>
       </c>
-      <c r="I7" s="102">
-        <v>0</v>
-      </c>
-      <c r="J7" s="102">
+      <c r="I7" s="96">
+        <v>0</v>
+      </c>
+      <c r="J7" s="96">
         <v>1</v>
       </c>
-      <c r="K7" s="102">
+      <c r="K7" s="96">
         <v>-1</v>
       </c>
-      <c r="L7" s="102">
+      <c r="L7" s="96">
         <v>1</v>
       </c>
-      <c r="M7" s="104"/>
+      <c r="M7" s="98"/>
     </row>
     <row r="8" spans="2:13">
-      <c r="B8" s="116" t="s">
+      <c r="B8" s="110" t="s">
         <v>219</v>
       </c>
-      <c r="C8" s="109">
+      <c r="C8" s="103">
         <v>6.4250000000000002E-3</v>
       </c>
-      <c r="D8" s="102">
+      <c r="D8" s="96">
         <v>800</v>
       </c>
-      <c r="E8" s="102"/>
-      <c r="F8" s="102">
+      <c r="E8" s="96"/>
+      <c r="F8" s="96">
         <v>2.0999999999999999E-3</v>
       </c>
-      <c r="G8" s="102">
+      <c r="G8" s="96">
         <v>0.8</v>
       </c>
-      <c r="H8" s="102">
+      <c r="H8" s="96">
         <v>0.8</v>
       </c>
-      <c r="I8" s="102">
-        <v>0</v>
-      </c>
-      <c r="J8" s="102">
+      <c r="I8" s="96">
+        <v>0</v>
+      </c>
+      <c r="J8" s="96">
         <v>-1</v>
       </c>
-      <c r="K8" s="102">
+      <c r="K8" s="96">
         <v>-1</v>
       </c>
-      <c r="L8" s="102">
+      <c r="L8" s="96">
         <v>1</v>
       </c>
-      <c r="M8" s="104"/>
+      <c r="M8" s="98"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="B9" s="116" t="s">
+      <c r="B9" s="110" t="s">
         <v>220</v>
       </c>
-      <c r="C9" s="109">
+      <c r="C9" s="103">
         <v>2.1919999999999999E-2</v>
       </c>
-      <c r="D9" s="102">
+      <c r="D9" s="96">
         <v>800</v>
       </c>
-      <c r="E9" s="102"/>
-      <c r="F9" s="102">
+      <c r="E9" s="96"/>
+      <c r="F9" s="96">
         <v>9.5999999999999992E-3</v>
       </c>
-      <c r="G9" s="102">
+      <c r="G9" s="96">
         <v>0.8</v>
       </c>
-      <c r="H9" s="102">
+      <c r="H9" s="96">
         <v>0.8</v>
       </c>
-      <c r="I9" s="102">
-        <v>0</v>
-      </c>
-      <c r="J9" s="102">
-        <v>0</v>
-      </c>
-      <c r="K9" s="102">
+      <c r="I9" s="96">
+        <v>0</v>
+      </c>
+      <c r="J9" s="96">
+        <v>0</v>
+      </c>
+      <c r="K9" s="96">
         <v>1</v>
       </c>
-      <c r="L9" s="102">
+      <c r="L9" s="96">
         <v>1</v>
       </c>
-      <c r="M9" s="104"/>
+      <c r="M9" s="98"/>
     </row>
     <row r="10" spans="2:13">
-      <c r="B10" s="116" t="s">
+      <c r="B10" s="110" t="s">
         <v>221</v>
       </c>
-      <c r="C10" s="109">
+      <c r="C10" s="103">
         <v>1.8E-3</v>
       </c>
-      <c r="D10" s="102">
+      <c r="D10" s="96">
         <v>800</v>
       </c>
-      <c r="E10" s="102"/>
-      <c r="F10" s="102">
+      <c r="E10" s="96"/>
+      <c r="F10" s="96">
         <v>5.7600000000000001E-4</v>
       </c>
-      <c r="G10" s="102">
+      <c r="G10" s="96">
         <v>0.8</v>
       </c>
-      <c r="H10" s="102">
+      <c r="H10" s="96">
         <v>0.8</v>
       </c>
-      <c r="I10" s="102">
-        <v>0</v>
-      </c>
-      <c r="J10" s="102">
-        <v>0</v>
-      </c>
-      <c r="K10" s="102">
+      <c r="I10" s="96">
+        <v>0</v>
+      </c>
+      <c r="J10" s="96">
+        <v>0</v>
+      </c>
+      <c r="K10" s="96">
         <v>1</v>
       </c>
-      <c r="L10" s="102">
+      <c r="L10" s="96">
         <v>1</v>
       </c>
-      <c r="M10" s="104"/>
+      <c r="M10" s="98"/>
     </row>
     <row r="11" spans="2:13">
-      <c r="B11" s="116" t="s">
+      <c r="B11" s="110" t="s">
         <v>222</v>
       </c>
-      <c r="C11" s="109">
+      <c r="C11" s="103">
         <v>1.8E-3</v>
       </c>
-      <c r="D11" s="102">
+      <c r="D11" s="96">
         <v>800</v>
       </c>
-      <c r="E11" s="102"/>
-      <c r="F11" s="102">
+      <c r="E11" s="96"/>
+      <c r="F11" s="96">
         <v>5.7600000000000001E-4</v>
       </c>
-      <c r="G11" s="102">
+      <c r="G11" s="96">
         <v>0.8</v>
       </c>
-      <c r="H11" s="102">
+      <c r="H11" s="96">
         <v>0.8</v>
       </c>
-      <c r="I11" s="102">
-        <v>0</v>
-      </c>
-      <c r="J11" s="102">
-        <v>0</v>
-      </c>
-      <c r="K11" s="102">
+      <c r="I11" s="96">
+        <v>0</v>
+      </c>
+      <c r="J11" s="96">
+        <v>0</v>
+      </c>
+      <c r="K11" s="96">
         <v>1</v>
       </c>
-      <c r="L11" s="102">
+      <c r="L11" s="96">
         <v>1</v>
       </c>
-      <c r="M11" s="104"/>
+      <c r="M11" s="98"/>
     </row>
     <row r="12" spans="2:13">
-      <c r="B12" s="116" t="s">
+      <c r="B12" s="110" t="s">
         <v>223</v>
       </c>
-      <c r="C12" s="109">
+      <c r="C12" s="103">
         <v>1.8E-3</v>
       </c>
-      <c r="D12" s="102">
+      <c r="D12" s="96">
         <v>800</v>
       </c>
-      <c r="E12" s="102"/>
-      <c r="F12" s="102">
+      <c r="E12" s="96"/>
+      <c r="F12" s="96">
         <v>5.7600000000000001E-4</v>
       </c>
-      <c r="G12" s="102">
+      <c r="G12" s="96">
         <v>0.8</v>
       </c>
-      <c r="H12" s="102">
+      <c r="H12" s="96">
         <v>0.8</v>
       </c>
-      <c r="I12" s="102">
-        <v>0</v>
-      </c>
-      <c r="J12" s="102">
-        <v>0</v>
-      </c>
-      <c r="K12" s="102">
+      <c r="I12" s="96">
+        <v>0</v>
+      </c>
+      <c r="J12" s="96">
+        <v>0</v>
+      </c>
+      <c r="K12" s="96">
         <v>1</v>
       </c>
-      <c r="L12" s="102">
+      <c r="L12" s="96">
         <v>1</v>
       </c>
-      <c r="M12" s="104"/>
+      <c r="M12" s="98"/>
     </row>
     <row r="13" spans="2:13">
-      <c r="B13" s="116" t="s">
+      <c r="B13" s="110" t="s">
         <v>224</v>
       </c>
-      <c r="C13" s="109">
+      <c r="C13" s="103">
         <v>1.8E-3</v>
       </c>
-      <c r="D13" s="102">
+      <c r="D13" s="96">
         <v>800</v>
       </c>
-      <c r="E13" s="102"/>
-      <c r="F13" s="102">
+      <c r="E13" s="96"/>
+      <c r="F13" s="96">
         <v>5.7600000000000001E-4</v>
       </c>
-      <c r="G13" s="102">
+      <c r="G13" s="96">
         <v>0.8</v>
       </c>
-      <c r="H13" s="102">
+      <c r="H13" s="96">
         <v>0.8</v>
       </c>
-      <c r="I13" s="102">
-        <v>0</v>
-      </c>
-      <c r="J13" s="102">
-        <v>0</v>
-      </c>
-      <c r="K13" s="102">
+      <c r="I13" s="96">
+        <v>0</v>
+      </c>
+      <c r="J13" s="96">
+        <v>0</v>
+      </c>
+      <c r="K13" s="96">
         <v>1</v>
       </c>
-      <c r="L13" s="102">
+      <c r="L13" s="96">
         <v>1</v>
       </c>
-      <c r="M13" s="104"/>
+      <c r="M13" s="98"/>
     </row>
     <row r="14" spans="2:13">
-      <c r="B14" s="116" t="s">
+      <c r="B14" s="110" t="s">
         <v>225</v>
       </c>
-      <c r="C14" s="109">
+      <c r="C14" s="103">
         <v>2.375E-2</v>
       </c>
-      <c r="D14" s="102">
+      <c r="D14" s="96">
         <v>600</v>
       </c>
-      <c r="E14" s="102"/>
-      <c r="F14" s="102">
+      <c r="E14" s="96"/>
+      <c r="F14" s="96">
         <v>0.01</v>
       </c>
-      <c r="G14" s="102"/>
-      <c r="H14" s="102"/>
-      <c r="I14" s="102"/>
-      <c r="J14" s="102"/>
-      <c r="K14" s="102"/>
-      <c r="L14" s="102">
-        <v>0</v>
-      </c>
-      <c r="M14" s="104"/>
+      <c r="G14" s="96"/>
+      <c r="H14" s="96"/>
+      <c r="I14" s="96"/>
+      <c r="J14" s="96"/>
+      <c r="K14" s="96"/>
+      <c r="L14" s="96">
+        <v>0</v>
+      </c>
+      <c r="M14" s="98"/>
     </row>
     <row r="15" spans="2:13">
-      <c r="B15" s="116" t="s">
+      <c r="B15" s="110" t="s">
         <v>226</v>
       </c>
-      <c r="C15" s="109">
+      <c r="C15" s="103">
         <v>0.125</v>
       </c>
-      <c r="D15" s="102">
+      <c r="D15" s="96">
         <v>800</v>
       </c>
-      <c r="E15" s="102"/>
-      <c r="F15" s="102">
+      <c r="E15" s="96"/>
+      <c r="F15" s="96">
         <v>0.01</v>
       </c>
-      <c r="G15" s="102"/>
-      <c r="H15" s="102"/>
-      <c r="I15" s="102"/>
-      <c r="J15" s="102"/>
-      <c r="K15" s="102"/>
-      <c r="L15" s="102">
-        <v>0</v>
-      </c>
-      <c r="M15" s="104"/>
+      <c r="G15" s="96"/>
+      <c r="H15" s="96"/>
+      <c r="I15" s="96"/>
+      <c r="J15" s="96"/>
+      <c r="K15" s="96"/>
+      <c r="L15" s="96">
+        <v>0</v>
+      </c>
+      <c r="M15" s="98"/>
     </row>
     <row r="16" spans="2:13">
-      <c r="B16" s="116" t="s">
+      <c r="B16" s="110" t="s">
         <v>227</v>
       </c>
-      <c r="C16" s="109">
+      <c r="C16" s="103">
         <v>3.9E-2</v>
       </c>
-      <c r="D16" s="102">
+      <c r="D16" s="96">
         <v>600</v>
       </c>
-      <c r="E16" s="102"/>
-      <c r="F16" s="102">
+      <c r="E16" s="96"/>
+      <c r="F16" s="96">
         <v>0.01</v>
       </c>
-      <c r="G16" s="102"/>
-      <c r="H16" s="102"/>
-      <c r="I16" s="102"/>
-      <c r="J16" s="102"/>
-      <c r="K16" s="102"/>
-      <c r="L16" s="102">
-        <v>0</v>
-      </c>
-      <c r="M16" s="104"/>
+      <c r="G16" s="96"/>
+      <c r="H16" s="96"/>
+      <c r="I16" s="96"/>
+      <c r="J16" s="96"/>
+      <c r="K16" s="96"/>
+      <c r="L16" s="96">
+        <v>0</v>
+      </c>
+      <c r="M16" s="98"/>
     </row>
     <row r="17" spans="2:13">
-      <c r="B17" s="116" t="s">
+      <c r="B17" s="110" t="s">
         <v>228</v>
       </c>
-      <c r="C17" s="109">
+      <c r="C17" s="103">
         <v>3.9E-2</v>
       </c>
-      <c r="D17" s="102">
+      <c r="D17" s="96">
         <v>600</v>
       </c>
-      <c r="E17" s="102"/>
-      <c r="F17" s="102">
+      <c r="E17" s="96"/>
+      <c r="F17" s="96">
         <v>0.1</v>
       </c>
-      <c r="G17" s="102"/>
-      <c r="H17" s="102"/>
-      <c r="I17" s="102"/>
-      <c r="J17" s="102"/>
-      <c r="K17" s="102"/>
-      <c r="L17" s="102">
-        <v>0</v>
-      </c>
-      <c r="M17" s="104"/>
+      <c r="G17" s="96"/>
+      <c r="H17" s="96"/>
+      <c r="I17" s="96"/>
+      <c r="J17" s="96"/>
+      <c r="K17" s="96"/>
+      <c r="L17" s="96">
+        <v>0</v>
+      </c>
+      <c r="M17" s="98"/>
     </row>
     <row r="18" spans="2:13">
-      <c r="B18" s="116" t="s">
+      <c r="B18" s="110" t="s">
         <v>229</v>
       </c>
-      <c r="C18" s="109">
+      <c r="C18" s="103">
         <v>3.9E-2</v>
       </c>
-      <c r="D18" s="102">
+      <c r="D18" s="96">
         <v>600</v>
       </c>
-      <c r="E18" s="102"/>
-      <c r="F18" s="102">
+      <c r="E18" s="96"/>
+      <c r="F18" s="96">
         <v>0.1</v>
       </c>
-      <c r="G18" s="102"/>
-      <c r="H18" s="102"/>
-      <c r="I18" s="102"/>
-      <c r="J18" s="102"/>
-      <c r="K18" s="102"/>
-      <c r="L18" s="102">
-        <v>0</v>
-      </c>
-      <c r="M18" s="104"/>
+      <c r="G18" s="96"/>
+      <c r="H18" s="96"/>
+      <c r="I18" s="96"/>
+      <c r="J18" s="96"/>
+      <c r="K18" s="96"/>
+      <c r="L18" s="96">
+        <v>0</v>
+      </c>
+      <c r="M18" s="98"/>
     </row>
     <row r="19" spans="2:13">
-      <c r="B19" s="116" t="s">
+      <c r="B19" s="110" t="s">
         <v>230</v>
       </c>
-      <c r="C19" s="109">
+      <c r="C19" s="103">
         <v>3.9E-2</v>
       </c>
-      <c r="D19" s="102">
+      <c r="D19" s="96">
         <v>600</v>
       </c>
-      <c r="E19" s="102"/>
-      <c r="F19" s="102">
+      <c r="E19" s="96"/>
+      <c r="F19" s="96">
         <v>0.1</v>
       </c>
-      <c r="G19" s="102"/>
-      <c r="H19" s="102"/>
-      <c r="I19" s="102"/>
-      <c r="J19" s="102"/>
-      <c r="K19" s="102"/>
-      <c r="L19" s="102">
-        <v>0</v>
-      </c>
-      <c r="M19" s="104"/>
+      <c r="G19" s="96"/>
+      <c r="H19" s="96"/>
+      <c r="I19" s="96"/>
+      <c r="J19" s="96"/>
+      <c r="K19" s="96"/>
+      <c r="L19" s="96">
+        <v>0</v>
+      </c>
+      <c r="M19" s="98"/>
     </row>
     <row r="20" spans="2:13">
-      <c r="B20" s="116" t="s">
+      <c r="B20" s="110" t="s">
         <v>231</v>
       </c>
-      <c r="C20" s="109">
+      <c r="C20" s="103">
         <v>0.05</v>
       </c>
-      <c r="D20" s="102">
+      <c r="D20" s="96">
         <v>600</v>
       </c>
-      <c r="E20" s="102"/>
-      <c r="F20" s="102">
+      <c r="E20" s="96"/>
+      <c r="F20" s="96">
         <v>0.1</v>
       </c>
-      <c r="G20" s="102"/>
-      <c r="H20" s="102"/>
-      <c r="I20" s="102"/>
-      <c r="J20" s="102"/>
-      <c r="K20" s="102"/>
-      <c r="L20" s="102">
-        <v>0</v>
-      </c>
-      <c r="M20" s="104"/>
+      <c r="G20" s="96"/>
+      <c r="H20" s="96"/>
+      <c r="I20" s="96"/>
+      <c r="J20" s="96"/>
+      <c r="K20" s="96"/>
+      <c r="L20" s="96">
+        <v>0</v>
+      </c>
+      <c r="M20" s="98"/>
     </row>
     <row r="21" spans="2:13">
-      <c r="B21" s="116" t="s">
+      <c r="B21" s="110" t="s">
         <v>232</v>
       </c>
-      <c r="C21" s="109">
+      <c r="C21" s="103">
         <v>0.05</v>
       </c>
-      <c r="D21" s="102">
+      <c r="D21" s="96">
         <v>600</v>
       </c>
-      <c r="E21" s="102"/>
-      <c r="F21" s="102">
+      <c r="E21" s="96"/>
+      <c r="F21" s="96">
         <v>0.1</v>
       </c>
-      <c r="G21" s="102"/>
-      <c r="H21" s="102"/>
-      <c r="I21" s="102"/>
-      <c r="J21" s="102"/>
-      <c r="K21" s="102"/>
-      <c r="L21" s="102">
-        <v>0</v>
-      </c>
-      <c r="M21" s="104"/>
+      <c r="G21" s="96"/>
+      <c r="H21" s="96"/>
+      <c r="I21" s="96"/>
+      <c r="J21" s="96"/>
+      <c r="K21" s="96"/>
+      <c r="L21" s="96">
+        <v>0</v>
+      </c>
+      <c r="M21" s="98"/>
     </row>
     <row r="22" spans="2:13">
-      <c r="B22" s="116" t="s">
+      <c r="B22" s="110" t="s">
         <v>233</v>
       </c>
-      <c r="C22" s="109">
+      <c r="C22" s="103">
         <v>3.8490000000000003E-2</v>
       </c>
-      <c r="D22" s="102">
+      <c r="D22" s="96">
         <v>600</v>
       </c>
-      <c r="E22" s="102"/>
-      <c r="F22" s="102">
+      <c r="E22" s="96"/>
+      <c r="F22" s="96">
         <v>8.6E-3</v>
       </c>
-      <c r="G22" s="102"/>
-      <c r="H22" s="102"/>
-      <c r="I22" s="102"/>
-      <c r="J22" s="102"/>
-      <c r="K22" s="102"/>
-      <c r="L22" s="102">
-        <v>0</v>
-      </c>
-      <c r="M22" s="104"/>
+      <c r="G22" s="96"/>
+      <c r="H22" s="96"/>
+      <c r="I22" s="96"/>
+      <c r="J22" s="96"/>
+      <c r="K22" s="96"/>
+      <c r="L22" s="96">
+        <v>0</v>
+      </c>
+      <c r="M22" s="98"/>
     </row>
     <row r="23" spans="2:13">
-      <c r="B23" s="116" t="s">
+      <c r="B23" s="110" t="s">
         <v>234</v>
       </c>
-      <c r="C23" s="109">
+      <c r="C23" s="103">
         <v>7.4999999999999997E-2</v>
       </c>
-      <c r="D23" s="102">
+      <c r="D23" s="96">
         <v>600</v>
       </c>
-      <c r="E23" s="102"/>
-      <c r="F23" s="102">
+      <c r="E23" s="96"/>
+      <c r="F23" s="96">
         <v>8.6E-3</v>
       </c>
-      <c r="G23" s="102"/>
-      <c r="H23" s="102"/>
-      <c r="I23" s="102"/>
-      <c r="J23" s="102"/>
-      <c r="K23" s="102"/>
-      <c r="L23" s="102">
-        <v>0</v>
-      </c>
-      <c r="M23" s="104"/>
+      <c r="G23" s="96"/>
+      <c r="H23" s="96"/>
+      <c r="I23" s="96"/>
+      <c r="J23" s="96"/>
+      <c r="K23" s="96"/>
+      <c r="L23" s="96">
+        <v>0</v>
+      </c>
+      <c r="M23" s="98"/>
     </row>
     <row r="24" spans="2:13">
-      <c r="B24" s="116" t="s">
+      <c r="B24" s="110" t="s">
         <v>235</v>
       </c>
-      <c r="C24" s="109">
+      <c r="C24" s="103">
         <v>8.5000000000000006E-2</v>
       </c>
-      <c r="D24" s="102">
+      <c r="D24" s="96">
         <v>600</v>
       </c>
-      <c r="E24" s="102">
+      <c r="E24" s="96">
         <v>15</v>
       </c>
-      <c r="F24" s="102">
+      <c r="F24" s="96">
         <v>0.08</v>
       </c>
-      <c r="G24" s="102"/>
-      <c r="H24" s="102"/>
-      <c r="I24" s="102"/>
-      <c r="J24" s="102"/>
-      <c r="K24" s="102"/>
-      <c r="L24" s="102">
-        <v>0</v>
-      </c>
-      <c r="M24" s="104">
+      <c r="G24" s="96"/>
+      <c r="H24" s="96"/>
+      <c r="I24" s="96"/>
+      <c r="J24" s="96"/>
+      <c r="K24" s="96"/>
+      <c r="L24" s="96">
+        <v>0</v>
+      </c>
+      <c r="M24" s="98">
         <v>0.7</v>
       </c>
     </row>
     <row r="25" spans="2:13">
-      <c r="B25" s="116" t="s">
+      <c r="B25" s="110" t="s">
         <v>236</v>
       </c>
-      <c r="C25" s="109">
+      <c r="C25" s="103">
         <v>2.4E-2</v>
       </c>
-      <c r="D25" s="102">
+      <c r="D25" s="96">
         <v>600</v>
       </c>
-      <c r="E25" s="102"/>
-      <c r="F25" s="102">
+      <c r="E25" s="96"/>
+      <c r="F25" s="96">
         <v>0.33</v>
       </c>
-      <c r="G25" s="102"/>
-      <c r="H25" s="102"/>
-      <c r="I25" s="102"/>
-      <c r="J25" s="102"/>
-      <c r="K25" s="102"/>
-      <c r="L25" s="102">
-        <v>0</v>
-      </c>
-      <c r="M25" s="104"/>
+      <c r="G25" s="96"/>
+      <c r="H25" s="96"/>
+      <c r="I25" s="96"/>
+      <c r="J25" s="96"/>
+      <c r="K25" s="96"/>
+      <c r="L25" s="96">
+        <v>0</v>
+      </c>
+      <c r="M25" s="98"/>
     </row>
     <row r="26" spans="2:13">
-      <c r="B26" s="116" t="s">
+      <c r="B26" s="110" t="s">
         <v>237</v>
       </c>
-      <c r="C26" s="109">
+      <c r="C26" s="103">
         <v>5.2999999999999999E-2</v>
       </c>
-      <c r="D26" s="102">
+      <c r="D26" s="96">
         <v>600</v>
       </c>
-      <c r="E26" s="102">
+      <c r="E26" s="96">
         <v>15</v>
       </c>
-      <c r="F26" s="102">
+      <c r="F26" s="96">
         <v>8.0940000000000005E-3</v>
       </c>
-      <c r="G26" s="102">
+      <c r="G26" s="96">
         <v>0.8</v>
       </c>
-      <c r="H26" s="102">
+      <c r="H26" s="96">
         <v>0.8</v>
       </c>
-      <c r="I26" s="102">
-        <v>0</v>
-      </c>
-      <c r="J26" s="102">
+      <c r="I26" s="96">
+        <v>0</v>
+      </c>
+      <c r="J26" s="96">
         <v>1</v>
       </c>
-      <c r="K26" s="102">
-        <v>0</v>
-      </c>
-      <c r="L26" s="102">
+      <c r="K26" s="96">
+        <v>0</v>
+      </c>
+      <c r="L26" s="96">
         <v>1</v>
       </c>
-      <c r="M26" s="104">
+      <c r="M26" s="98">
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
     <row r="27" spans="2:13">
-      <c r="B27" s="116" t="s">
+      <c r="B27" s="110" t="s">
         <v>238</v>
       </c>
-      <c r="C27" s="109">
+      <c r="C27" s="103">
         <v>4.3999999999999997E-2</v>
       </c>
-      <c r="D27" s="102">
+      <c r="D27" s="96">
         <v>600</v>
       </c>
-      <c r="E27" s="102">
+      <c r="E27" s="96">
         <v>15</v>
       </c>
-      <c r="F27" s="102">
+      <c r="F27" s="96">
         <v>8.0940000000000005E-3</v>
       </c>
-      <c r="G27" s="102">
+      <c r="G27" s="96">
         <v>0.8</v>
       </c>
-      <c r="H27" s="102">
+      <c r="H27" s="96">
         <v>0.8</v>
       </c>
-      <c r="I27" s="102">
-        <v>0</v>
-      </c>
-      <c r="J27" s="102">
+      <c r="I27" s="96">
+        <v>0</v>
+      </c>
+      <c r="J27" s="96">
         <v>-1</v>
       </c>
-      <c r="K27" s="102">
-        <v>0</v>
-      </c>
-      <c r="L27" s="102">
+      <c r="K27" s="96">
+        <v>0</v>
+      </c>
+      <c r="L27" s="96">
         <v>1</v>
       </c>
-      <c r="M27" s="104">
+      <c r="M27" s="98">
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
     <row r="28" spans="2:13">
-      <c r="B28" s="116" t="s">
+      <c r="B28" s="110" t="s">
         <v>239</v>
       </c>
-      <c r="C28" s="109">
+      <c r="C28" s="103">
         <v>4.4999999999999998E-2</v>
       </c>
-      <c r="D28" s="102">
+      <c r="D28" s="96">
         <v>600</v>
       </c>
-      <c r="E28" s="102">
+      <c r="E28" s="96">
         <v>15</v>
       </c>
-      <c r="F28" s="102">
+      <c r="F28" s="96">
         <v>8.0940000000000005E-3</v>
       </c>
-      <c r="G28" s="102">
+      <c r="G28" s="96">
         <v>0.8</v>
       </c>
-      <c r="H28" s="102">
+      <c r="H28" s="96">
         <v>0.8</v>
       </c>
-      <c r="I28" s="102">
+      <c r="I28" s="96">
         <v>1</v>
       </c>
-      <c r="J28" s="102">
-        <v>0</v>
-      </c>
-      <c r="K28" s="102">
-        <v>0</v>
-      </c>
-      <c r="L28" s="102">
+      <c r="J28" s="96">
+        <v>0</v>
+      </c>
+      <c r="K28" s="96">
+        <v>0</v>
+      </c>
+      <c r="L28" s="96">
         <v>1</v>
       </c>
-      <c r="M28" s="104">
+      <c r="M28" s="98">
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
     <row r="29" spans="2:13">
-      <c r="B29" s="116" t="s">
+      <c r="B29" s="110" t="s">
         <v>240</v>
       </c>
-      <c r="C29" s="109">
+      <c r="C29" s="103">
         <v>5.2999999999999999E-2</v>
       </c>
-      <c r="D29" s="102">
+      <c r="D29" s="96">
         <v>600</v>
       </c>
-      <c r="E29" s="102">
+      <c r="E29" s="96">
         <v>15</v>
       </c>
-      <c r="F29" s="102">
+      <c r="F29" s="96">
         <v>8.0940000000000005E-3</v>
       </c>
-      <c r="G29" s="102">
+      <c r="G29" s="96">
         <v>0.8</v>
       </c>
-      <c r="H29" s="102">
+      <c r="H29" s="96">
         <v>0.8</v>
       </c>
-      <c r="I29" s="102">
+      <c r="I29" s="96">
         <v>-1</v>
       </c>
-      <c r="J29" s="102">
-        <v>0</v>
-      </c>
-      <c r="K29" s="102">
-        <v>0</v>
-      </c>
-      <c r="L29" s="102">
+      <c r="J29" s="96">
+        <v>0</v>
+      </c>
+      <c r="K29" s="96">
+        <v>0</v>
+      </c>
+      <c r="L29" s="96">
         <v>1</v>
       </c>
-      <c r="M29" s="104">
+      <c r="M29" s="98">
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
     <row r="30" spans="2:13">
-      <c r="B30" s="116" t="s">
+      <c r="B30" s="110" t="s">
         <v>241</v>
       </c>
-      <c r="C30" s="109">
+      <c r="C30" s="103">
         <v>5.7500000000000002E-2</v>
       </c>
-      <c r="D30" s="102">
+      <c r="D30" s="96">
         <v>600</v>
       </c>
-      <c r="E30" s="102">
+      <c r="E30" s="96">
         <v>15</v>
       </c>
-      <c r="F30" s="102">
+      <c r="F30" s="96">
         <v>8.4469999999999996E-3</v>
       </c>
-      <c r="G30" s="102">
+      <c r="G30" s="96">
         <v>0.8</v>
       </c>
-      <c r="H30" s="102">
+      <c r="H30" s="96">
         <v>0.8</v>
       </c>
-      <c r="I30" s="102">
-        <v>0</v>
-      </c>
-      <c r="J30" s="102">
-        <v>0</v>
-      </c>
-      <c r="K30" s="102">
+      <c r="I30" s="96">
+        <v>0</v>
+      </c>
+      <c r="J30" s="96">
+        <v>0</v>
+      </c>
+      <c r="K30" s="96">
         <v>-1</v>
       </c>
-      <c r="L30" s="102">
+      <c r="L30" s="96">
         <v>1</v>
       </c>
-      <c r="M30" s="104">
+      <c r="M30" s="98">
         <v>2.2000000000000001E-3</v>
       </c>
     </row>
     <row r="31" spans="2:13" ht="15.75" thickBot="1">
-      <c r="B31" s="117" t="s">
+      <c r="B31" s="111" t="s">
         <v>242</v>
       </c>
-      <c r="C31" s="110">
+      <c r="C31" s="104">
         <v>0.04</v>
       </c>
-      <c r="D31" s="103">
+      <c r="D31" s="97">
         <v>600</v>
       </c>
-      <c r="E31" s="103"/>
-      <c r="F31" s="103">
+      <c r="E31" s="97"/>
+      <c r="F31" s="97">
         <v>0.01</v>
       </c>
-      <c r="G31" s="103"/>
-      <c r="H31" s="103"/>
-      <c r="I31" s="103"/>
-      <c r="J31" s="103"/>
-      <c r="K31" s="103"/>
-      <c r="L31" s="103">
-        <v>0</v>
-      </c>
-      <c r="M31" s="105"/>
+      <c r="G31" s="97"/>
+      <c r="H31" s="97"/>
+      <c r="I31" s="97"/>
+      <c r="J31" s="97"/>
+      <c r="K31" s="97"/>
+      <c r="L31" s="97">
+        <v>0</v>
+      </c>
+      <c r="M31" s="99"/>
     </row>
     <row r="32" spans="2:13">
       <c r="B32" s="80"/>

</xml_diff>

<commit_message>
Orbit and orientation overhaul.
Added the posibility to define orbit and orientation from the excel.
</commit_message>
<xml_diff>
--- a/teidecode_v1/Thermal_Data.xlsx
+++ b/teidecode_v1/Thermal_Data.xlsx
@@ -8,18 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Eduardo Navarro\Desktop\Cosas\Teidesat\Nueva carpeta\TeideThermal\teidecode_v1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DB26D28-3013-4CD9-BC48-2EE9A94F7B00}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{96163878-F97A-42E9-BAD0-A61ED876CF6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="1" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Nodes properties" sheetId="1" r:id="rId1"/>
     <sheet name="Conductances determination" sheetId="3" r:id="rId2"/>
-    <sheet name="Startup Parameters" sheetId="7" r:id="rId3"/>
-    <sheet name="Operation" sheetId="5" r:id="rId4"/>
-    <sheet name="Modes" sheetId="6" r:id="rId5"/>
-    <sheet name="Nodes thermal properties" sheetId="4" r:id="rId6"/>
-    <sheet name="Conductances_between_nodes" sheetId="2" r:id="rId7"/>
+    <sheet name="Orbital Parameters" sheetId="8" r:id="rId3"/>
+    <sheet name="Startup Parameters" sheetId="7" r:id="rId4"/>
+    <sheet name="Operation" sheetId="5" r:id="rId5"/>
+    <sheet name="Modes" sheetId="6" r:id="rId6"/>
+    <sheet name="Nodes thermal properties" sheetId="4" r:id="rId7"/>
+    <sheet name="Conductances_between_nodes" sheetId="2" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -35,7 +36,7 @@
       </xcalcf:calcFeatures>
     </ext>
     <ext uri="GoogleSheetsCustomDataVersion1">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId8" roundtripDataSignature="AMtx7mjKFLR0Am3JTZ+8bb0VcOSu/VdiBw=="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataSignature="AMtx7mjKFLR0Am3JTZ+8bb0VcOSu/VdiBw=="/>
     </ext>
   </extLst>
 </workbook>
@@ -457,7 +458,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="787" uniqueCount="268">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="793" uniqueCount="274">
   <si>
     <t>Esta tabla representado el struct con todos los datos de entrada que uso para el satélite,¿que le falta? pues el coeficiente Cp (specific heat capacity ) esta bastamente aproximado y habría que mirar material por material, puede que algo de info útil pueda ser encontrada en la tabla de mecánica</t>
   </si>
@@ -1263,6 +1264,24 @@
   <si>
     <t>Radiation to enviroment (1=Yes, 0=No)</t>
   </si>
+  <si>
+    <t>Yaw</t>
+  </si>
+  <si>
+    <t>Pitch</t>
+  </si>
+  <si>
+    <t>Roll</t>
+  </si>
+  <si>
+    <t>Longitude of ascending node</t>
+  </si>
+  <si>
+    <t>Inclination</t>
+  </si>
+  <si>
+    <t>Orbital height (Km)</t>
+  </si>
 </sst>
 </file>
 
@@ -1274,11 +1293,32 @@
     <numFmt numFmtId="166" formatCode="#,##0.000000"/>
     <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
-  <fonts count="12">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -1353,7 +1393,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="22">
+  <fills count="23">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1477,6 +1517,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.39997558519241921"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.39997558519241921"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -2290,163 +2336,163 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="146">
+  <cellXfs count="152">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" quotePrefix="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="9" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="5" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
-    <xf numFmtId="165" fontId="9" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="165" fontId="12" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="10" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="11" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="7" fillId="12" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="2" fontId="5" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="2" fontId="8" fillId="15" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="15" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="166" fontId="5" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="17" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="167" fontId="5" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="167" fontId="8" fillId="9" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="5" fillId="14" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="8" fillId="14" borderId="14" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="13" fillId="16" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="16" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="13" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="13" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="49" fontId="4" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="164" fontId="4" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="13" borderId="0" xfId="0" quotePrefix="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="49" fontId="7" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="164" fontId="7" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2458,13 +2504,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2492,13 +2538,13 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="49" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="48" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -2507,7 +2553,7 @@
     <xf numFmtId="0" fontId="0" fillId="19" borderId="50" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="36" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="19" borderId="37" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="17" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="17" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="52" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2516,17 +2562,17 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="53" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="53" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="54" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="42" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" xfId="0" applyBorder="1" applyAlignment="1">
@@ -2562,41 +2608,53 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="59" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="19" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="20" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="43" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="40" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="18" borderId="57" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="21" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="21" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="38" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="19" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="22" borderId="55" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="28" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -9988,10 +10046,10 @@
         <v>149</v>
       </c>
       <c r="G2" s="32"/>
-      <c r="H2" s="140" t="s">
+      <c r="H2" s="145" t="s">
         <v>150</v>
       </c>
-      <c r="I2" s="141"/>
+      <c r="I2" s="146"/>
     </row>
     <row r="3" spans="1:9">
       <c r="A3" s="33" t="s">
@@ -10993,6 +11051,63 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{20E01517-96A7-414C-8030-8BA1AC45135C}">
+  <dimension ref="B1:G5"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
+  <cols>
+    <col min="5" max="5" width="16" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:7" ht="15.75" thickBot="1"/>
+    <row r="2" spans="2:7" ht="37.5" customHeight="1">
+      <c r="B2" s="148" t="s">
+        <v>268</v>
+      </c>
+      <c r="C2" s="149" t="s">
+        <v>269</v>
+      </c>
+      <c r="D2" s="149" t="s">
+        <v>270</v>
+      </c>
+      <c r="E2" s="149" t="s">
+        <v>271</v>
+      </c>
+      <c r="F2" s="149" t="s">
+        <v>272</v>
+      </c>
+      <c r="G2" s="150" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="3" spans="2:7" ht="15.75" thickBot="1">
+      <c r="B3" s="151">
+        <v>0</v>
+      </c>
+      <c r="C3" s="97">
+        <v>0</v>
+      </c>
+      <c r="D3" s="97">
+        <v>0</v>
+      </c>
+      <c r="E3" s="97">
+        <v>0</v>
+      </c>
+      <c r="F3" s="97">
+        <v>0</v>
+      </c>
+      <c r="G3" s="99">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7">
+      <c r="B5" s="147"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3AFF58F4-2122-4D7A-8536-BCD5250BA286}">
   <dimension ref="B1:F3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
@@ -11044,7 +11159,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4723E147-5D28-48F2-9A19-B61306348D73}">
   <dimension ref="A1:N37"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
@@ -11057,16 +11172,16 @@
       <c r="B2" s="132" t="s">
         <v>257</v>
       </c>
-      <c r="C2" s="142" t="s">
+      <c r="C2" s="143" t="s">
+        <v>260</v>
+      </c>
+      <c r="D2" s="141" t="s">
         <v>259</v>
       </c>
-      <c r="D2" s="144" t="s">
-        <v>259</v>
-      </c>
-      <c r="E2" s="144" t="s">
+      <c r="E2" s="141" t="s">
         <v>258</v>
       </c>
-      <c r="F2" s="145" t="s">
+      <c r="F2" s="142" t="s">
         <v>260</v>
       </c>
       <c r="G2" s="117"/>
@@ -11077,19 +11192,19 @@
       </c>
       <c r="C3" s="89">
         <f>IFERROR(C4+C5*60+C6*3600+C7*3600*24+B3,C4+C5*60+C6*3600+C7*3600*24)</f>
-        <v>32400</v>
+        <v>25200</v>
       </c>
       <c r="D3" s="89">
         <f t="shared" ref="D3:F3" si="0">IFERROR(D4+D5*60+D6*3600+D7*3600*24+C3,D4+D5*60+D6*3600+D7*3600*24)</f>
-        <v>32400</v>
+        <v>25200</v>
       </c>
       <c r="E3" s="89">
         <f t="shared" si="0"/>
-        <v>32400</v>
+        <v>25200</v>
       </c>
       <c r="F3" s="89">
         <f t="shared" si="0"/>
-        <v>32460</v>
+        <v>25200</v>
       </c>
       <c r="G3" s="91"/>
       <c r="H3" s="81"/>
@@ -11116,29 +11231,35 @@
       </c>
       <c r="C5" s="86"/>
       <c r="D5" s="84"/>
-      <c r="E5" s="83"/>
-      <c r="F5" s="90">
-        <v>1</v>
-      </c>
+      <c r="E5" s="83">
+        <v>0</v>
+      </c>
+      <c r="F5" s="90"/>
       <c r="G5" s="91"/>
     </row>
     <row r="6" spans="1:14">
       <c r="B6" s="88" t="s">
         <v>254</v>
       </c>
-      <c r="C6" s="143">
-        <v>9</v>
-      </c>
-      <c r="D6" s="84"/>
+      <c r="C6" s="140">
+        <v>7</v>
+      </c>
+      <c r="D6" s="84">
+        <v>0</v>
+      </c>
       <c r="E6" s="83"/>
-      <c r="F6" s="90"/>
+      <c r="F6" s="90">
+        <v>0</v>
+      </c>
       <c r="G6" s="91"/>
     </row>
     <row r="7" spans="1:14">
       <c r="B7" s="112" t="s">
         <v>261</v>
       </c>
-      <c r="C7" s="113"/>
+      <c r="C7" s="113">
+        <v>0</v>
+      </c>
       <c r="D7" s="114"/>
       <c r="E7" s="115"/>
       <c r="F7" s="116"/>
@@ -11364,7 +11485,7 @@
       </c>
       <c r="C15" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A15+1,FALSE)</f>
-        <v>5.0999999999999996</v>
+        <v>0</v>
       </c>
       <c r="D15" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A15+1,FALSE)</f>
@@ -11394,7 +11515,7 @@
       </c>
       <c r="C16" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A16+1,FALSE)</f>
-        <v>5.0999999999999996</v>
+        <v>0</v>
       </c>
       <c r="D16" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A16+1,FALSE)</f>
@@ -11424,7 +11545,7 @@
       </c>
       <c r="C17" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A17+1,FALSE)</f>
-        <v>5.0999999999999996</v>
+        <v>0</v>
       </c>
       <c r="D17" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A17+1,FALSE)</f>
@@ -11454,7 +11575,7 @@
       </c>
       <c r="C18" s="93">
         <f>HLOOKUP(C$2,Modes!$B$2:$O$31,$A18+1,FALSE)</f>
-        <v>5.0999999999999996</v>
+        <v>0</v>
       </c>
       <c r="D18" s="93">
         <f>HLOOKUP(D$2,Modes!$B$2:$O$31,$A18+1,FALSE)</f>
@@ -12022,7 +12143,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B005E130-2D16-4A0C-8BB3-2172273CEA1D}">
   <dimension ref="B1:O32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
@@ -12772,7 +12893,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4985A03E-5096-4337-92A3-24224C69AEFA}">
   <dimension ref="B1:M32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15"/>
@@ -12920,10 +13041,10 @@
         <v>0</v>
       </c>
       <c r="J5" s="96">
-        <v>-1</v>
+        <v>-0.70709999999999995</v>
       </c>
       <c r="K5" s="96">
-        <v>1</v>
+        <v>0.70709999999999995</v>
       </c>
       <c r="L5" s="96">
         <v>1</v>
@@ -12954,10 +13075,10 @@
         <v>0</v>
       </c>
       <c r="J6" s="96">
-        <v>1</v>
+        <v>0.70709999999999995</v>
       </c>
       <c r="K6" s="96">
-        <v>1</v>
+        <v>0.70709999999999995</v>
       </c>
       <c r="L6" s="96">
         <v>1</v>
@@ -12988,10 +13109,10 @@
         <v>0</v>
       </c>
       <c r="J7" s="96">
-        <v>1</v>
+        <v>0.70709999999999995</v>
       </c>
       <c r="K7" s="96">
-        <v>-1</v>
+        <v>-0.70709999999999995</v>
       </c>
       <c r="L7" s="96">
         <v>1</v>
@@ -13022,10 +13143,10 @@
         <v>0</v>
       </c>
       <c r="J8" s="96">
-        <v>-1</v>
+        <v>-0.70709999999999995</v>
       </c>
       <c r="K8" s="96">
-        <v>-1</v>
+        <v>-0.70709999999999995</v>
       </c>
       <c r="L8" s="96">
         <v>1</v>
@@ -13033,7 +13154,7 @@
       <c r="M8" s="98"/>
     </row>
     <row r="9" spans="2:13">
-      <c r="B9" s="110" t="s">
+      <c r="B9" s="144" t="s">
         <v>220</v>
       </c>
       <c r="C9" s="103">
@@ -13716,7 +13837,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:AD990"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>

</xml_diff>